<commit_message>
Allow saving incomplete contracts, editing paid dates, update Excel template
- New/edit contract form: only ФИО клиента is required now to enable
  the save button, matching the already-relaxed Excel import rules;
  term defaults to 1 month when left blank instead of blocking save
- Payments that are already marked paid can have their date corrected
  via a new "изменить дату" (pencil) button next to "Отменить",
  reusing the inline date picker in an "edit" mode instead of only
  allowing undo + re-pay
- Excel template: added a "Комментарий" column to Договоры (imported
  into the new comment field), reworded the Инструкция sheet to match
  the relaxed required-fields rule, and one example row now
  demonstrates leaving price/term blank

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/rassrochki_template.xlsx
+++ b/public/rassrochki_template.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B39"/>
+  <dimension ref="B2:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -561,193 +561,214 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>• Обязательные поля в «Договоры»: ФИО клиента, Цена товара, Срок (мес).</t>
+          <t>• В «Договоры» обязательно только ФИО клиента — остальные поля можно оставить</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>• «Наценка, %» — впишите процент, и колонка «Наценка, ₽» рассчитает сумму</t>
+          <t xml:space="preserve">   пустыми, если информация ещё не известна (например, точная цена или срок),</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   автоматически по формуле (принцип как на сайте: меняете цену/взнос —</t>
+          <t xml:space="preserve">   и дозаполнить их позже прямо на сайте кнопкой «Изменить договор».</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   сумма наценки пересчитывается).</t>
+          <t>• «Наценка, %» — впишите процент, и колонка «Наценка, ₽» рассчитает сумму</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>• Если удобнее задать наценку сразу в рублях — сотрите формулу в ячейке</t>
+          <t xml:space="preserve">   автоматически по формуле (принцип как на сайте: меняете цену/взнос —</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   «Наценка, ₽» и впишите число вручную (процент в этой строке можно</t>
+          <t xml:space="preserve">   сумма наценки пересчитывается).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   оставить пустым). При загрузке на сайт используется то значение,</t>
+          <t>• Если удобнее задать наценку сразу в рублях — сотрите формулу в ячейке</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   которое реально стоит в ячейке — формула это или вручную введённое число,</t>
+          <t xml:space="preserve">   «Наценка, ₽» и впишите число вручную (процент в этой строке можно</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   неважно.</t>
+          <t xml:space="preserve">   оставить пустым). При загрузке на сайт используется то значение,</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>• «Источник финансирования» — впишите имя вкладчика точно как во вкладке</t>
+          <t xml:space="preserve">   которое реально стоит в ячейке — формула это или вручную введённое число,</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   «Вкладчики» (есть выпадающий список), либо оставьте пустым — тогда договор</t>
+          <t xml:space="preserve">   неважно.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   попадёт в «Общий пул» (без привязки к конкретному вкладчику).</t>
+          <t>• «Источник финансирования» — впишите имя вкладчика точно как во вкладке</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>• «Дата 1-го платежа» — дата в формате ДД.ММ.ГГГГ.</t>
+          <t xml:space="preserve">   «Вкладчики» (есть выпадающий список), либо оставьте пустым — тогда договор</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>• Строки-примеры выделены курсивом — их можно удалить перед загрузкой.</t>
+          <t xml:space="preserve">   попадёт в «Общий пул» (без привязки к конкретному вкладчику).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>• «Дата 1-го платежа» — дата в формате ДД.ММ.ГГГГ.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Вкладка «Платежи» — если по договору уже что-то оплачено:</t>
+          <t>• «Комментарий» — необязательное поле, любая заметка по договору.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>• По одной строке на каждый оплаченный платёж: ФИО клиента, № платежа</t>
+          <t>• Строки-примеры выделены курсивом — их можно удалить перед загрузкой.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   по графику (1 — первый платёж, 2 — второй и т.д.) и дата, когда он</t>
-        </is>
-      </c>
+      <c r="B28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   был реально оплачен.</t>
+          <t>Вкладка «Платежи» — если по договору уже что-то оплачено:</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>• Колонку «Товар» заполняйте, только если у клиента несколько договоров —</t>
+          <t>• По одной строке на каждый оплаченный платёж: ФИО клиента, № платежа</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   она нужна, чтобы отличить, к какому именно договору относится платёж.</t>
+          <t xml:space="preserve">   по графику (1 — первый платёж, 2 — второй и т.д.) и дата, когда он</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>• Не оплаченные платежи вносить не нужно — про них ничего писать не надо,</t>
+          <t xml:space="preserve">   был реально оплачен.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   на сайте они и так будут отображаться как «Ожидает» / «Просрочен».</t>
+          <t>• Колонку «Товар» заполняйте, только если у клиента несколько договоров —</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>• Эта вкладка также работает при повторной загрузке — можно отмечать оплаты</t>
+          <t xml:space="preserve">   она нужна, чтобы отличить, к какому именно договору относится платёж.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   и по договорам, которые уже были на сайте раньше (по ФИО и, если нужно,</t>
+          <t>• Не оплаченные платежи вносить не нужно — про них ничего писать не надо,</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   товару).</t>
+          <t xml:space="preserve">   на сайте они и так будут отображаться как «Ожидает» / «Просрочен».</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>• Эта вкладка также работает при повторной загрузке — можно отмечать оплаты</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Повторная загрузка не удаляет уже имеющиеся на сайте данные — новые вкладчики,</t>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   и по договорам, которые уже были на сайте раньше (по ФИО и, если нужно,</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   товару).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Повторная загрузка не удаляет уже имеющиеся на сайте данные — новые вкладчики,</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>договоры и платежи из файла добавляются к существующим.</t>
         </is>
@@ -918,7 +939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J200"/>
+  <dimension ref="A1:K200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -931,6 +952,7 @@
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -984,6 +1006,11 @@
           <t>Источник финансирования</t>
         </is>
       </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -1018,11 +1045,16 @@
         <v>6</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="J2" s="9" t="inlineStr">
         <is>
           <t>Иванов Пётр</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>Просил напомнить за неделю до платежа</t>
         </is>
       </c>
     </row>
@@ -1042,23 +1074,18 @@
           <t>Стиральная машина</t>
         </is>
       </c>
-      <c r="D3" s="10" t="n">
-        <v>60000</v>
-      </c>
-      <c r="E3" s="10" t="n">
-        <v>10000</v>
-      </c>
+      <c r="D3" s="10" t="inlineStr"/>
+      <c r="E3" s="10" t="inlineStr"/>
       <c r="F3" s="11" t="n"/>
       <c r="G3" s="10" t="n">
         <v>8000</v>
       </c>
-      <c r="H3" s="9" t="n">
-        <v>5</v>
-      </c>
+      <c r="H3" s="9" t="inlineStr"/>
       <c r="I3" s="12" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="J3" s="9" t="n"/>
+      <c r="K3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n"/>
@@ -1074,6 +1101,7 @@
       <c r="H4" s="7" t="n"/>
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>
@@ -1089,6 +1117,7 @@
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="14" t="n"/>
       <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n"/>
@@ -1104,6 +1133,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="14" t="n"/>
       <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -1119,6 +1149,7 @@
       <c r="H7" s="7" t="n"/>
       <c r="I7" s="14" t="n"/>
       <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n"/>
@@ -1134,6 +1165,7 @@
       <c r="H8" s="7" t="n"/>
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -1149,6 +1181,7 @@
       <c r="H9" s="7" t="n"/>
       <c r="I9" s="14" t="n"/>
       <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -1164,6 +1197,7 @@
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -1179,6 +1213,7 @@
       <c r="H11" s="7" t="n"/>
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="7" t="n"/>
+      <c r="K11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -1194,6 +1229,7 @@
       <c r="H12" s="7" t="n"/>
       <c r="I12" s="14" t="n"/>
       <c r="J12" s="7" t="n"/>
+      <c r="K12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -1209,6 +1245,7 @@
       <c r="H13" s="7" t="n"/>
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1224,6 +1261,7 @@
       <c r="H14" s="7" t="n"/>
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1239,6 +1277,7 @@
       <c r="H15" s="7" t="n"/>
       <c r="I15" s="14" t="n"/>
       <c r="J15" s="7" t="n"/>
+      <c r="K15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -1254,6 +1293,7 @@
       <c r="H16" s="7" t="n"/>
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="7" t="n"/>
+      <c r="K16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1269,6 +1309,7 @@
       <c r="H17" s="7" t="n"/>
       <c r="I17" s="14" t="n"/>
       <c r="J17" s="7" t="n"/>
+      <c r="K17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1284,6 +1325,7 @@
       <c r="H18" s="7" t="n"/>
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -1299,6 +1341,7 @@
       <c r="H19" s="7" t="n"/>
       <c r="I19" s="14" t="n"/>
       <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -1314,6 +1357,7 @@
       <c r="H20" s="7" t="n"/>
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="7" t="n"/>
+      <c r="K20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -1329,6 +1373,7 @@
       <c r="H21" s="7" t="n"/>
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="7" t="n"/>
+      <c r="K21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -1344,6 +1389,7 @@
       <c r="H22" s="7" t="n"/>
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="7" t="n"/>
+      <c r="K22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -1359,6 +1405,7 @@
       <c r="H23" s="7" t="n"/>
       <c r="I23" s="14" t="n"/>
       <c r="J23" s="7" t="n"/>
+      <c r="K23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -1374,6 +1421,7 @@
       <c r="H24" s="7" t="n"/>
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="7" t="n"/>
+      <c r="K24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -1389,6 +1437,7 @@
       <c r="H25" s="7" t="n"/>
       <c r="I25" s="14" t="n"/>
       <c r="J25" s="7" t="n"/>
+      <c r="K25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -1404,6 +1453,7 @@
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="7" t="n"/>
+      <c r="K26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -1419,6 +1469,7 @@
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="14" t="n"/>
       <c r="J27" s="7" t="n"/>
+      <c r="K27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -1434,6 +1485,7 @@
       <c r="H28" s="7" t="n"/>
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="7" t="n"/>
+      <c r="K28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -1449,6 +1501,7 @@
       <c r="H29" s="7" t="n"/>
       <c r="I29" s="14" t="n"/>
       <c r="J29" s="7" t="n"/>
+      <c r="K29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -1464,6 +1517,7 @@
       <c r="H30" s="7" t="n"/>
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="7" t="n"/>
+      <c r="K30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -1479,6 +1533,7 @@
       <c r="H31" s="7" t="n"/>
       <c r="I31" s="14" t="n"/>
       <c r="J31" s="7" t="n"/>
+      <c r="K31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -1494,6 +1549,7 @@
       <c r="H32" s="7" t="n"/>
       <c r="I32" s="14" t="n"/>
       <c r="J32" s="7" t="n"/>
+      <c r="K32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -1509,6 +1565,7 @@
       <c r="H33" s="7" t="n"/>
       <c r="I33" s="14" t="n"/>
       <c r="J33" s="7" t="n"/>
+      <c r="K33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -1524,6 +1581,7 @@
       <c r="H34" s="7" t="n"/>
       <c r="I34" s="14" t="n"/>
       <c r="J34" s="7" t="n"/>
+      <c r="K34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -1539,6 +1597,7 @@
       <c r="H35" s="7" t="n"/>
       <c r="I35" s="14" t="n"/>
       <c r="J35" s="7" t="n"/>
+      <c r="K35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -1554,6 +1613,7 @@
       <c r="H36" s="7" t="n"/>
       <c r="I36" s="14" t="n"/>
       <c r="J36" s="7" t="n"/>
+      <c r="K36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -1569,6 +1629,7 @@
       <c r="H37" s="7" t="n"/>
       <c r="I37" s="14" t="n"/>
       <c r="J37" s="7" t="n"/>
+      <c r="K37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -1584,6 +1645,7 @@
       <c r="H38" s="7" t="n"/>
       <c r="I38" s="14" t="n"/>
       <c r="J38" s="7" t="n"/>
+      <c r="K38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
@@ -1599,6 +1661,7 @@
       <c r="H39" s="7" t="n"/>
       <c r="I39" s="14" t="n"/>
       <c r="J39" s="7" t="n"/>
+      <c r="K39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n"/>
@@ -1614,6 +1677,7 @@
       <c r="H40" s="7" t="n"/>
       <c r="I40" s="14" t="n"/>
       <c r="J40" s="7" t="n"/>
+      <c r="K40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n"/>
@@ -1629,6 +1693,7 @@
       <c r="H41" s="7" t="n"/>
       <c r="I41" s="14" t="n"/>
       <c r="J41" s="7" t="n"/>
+      <c r="K41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n"/>
@@ -1644,6 +1709,7 @@
       <c r="H42" s="7" t="n"/>
       <c r="I42" s="14" t="n"/>
       <c r="J42" s="7" t="n"/>
+      <c r="K42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n"/>
@@ -1659,6 +1725,7 @@
       <c r="H43" s="7" t="n"/>
       <c r="I43" s="14" t="n"/>
       <c r="J43" s="7" t="n"/>
+      <c r="K43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n"/>
@@ -1674,6 +1741,7 @@
       <c r="H44" s="7" t="n"/>
       <c r="I44" s="14" t="n"/>
       <c r="J44" s="7" t="n"/>
+      <c r="K44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n"/>
@@ -1689,6 +1757,7 @@
       <c r="H45" s="7" t="n"/>
       <c r="I45" s="14" t="n"/>
       <c r="J45" s="7" t="n"/>
+      <c r="K45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n"/>
@@ -1704,6 +1773,7 @@
       <c r="H46" s="7" t="n"/>
       <c r="I46" s="14" t="n"/>
       <c r="J46" s="7" t="n"/>
+      <c r="K46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n"/>
@@ -1719,6 +1789,7 @@
       <c r="H47" s="7" t="n"/>
       <c r="I47" s="14" t="n"/>
       <c r="J47" s="7" t="n"/>
+      <c r="K47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -1734,6 +1805,7 @@
       <c r="H48" s="7" t="n"/>
       <c r="I48" s="14" t="n"/>
       <c r="J48" s="7" t="n"/>
+      <c r="K48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n"/>
@@ -1749,6 +1821,7 @@
       <c r="H49" s="7" t="n"/>
       <c r="I49" s="14" t="n"/>
       <c r="J49" s="7" t="n"/>
+      <c r="K49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n"/>
@@ -1764,6 +1837,7 @@
       <c r="H50" s="7" t="n"/>
       <c r="I50" s="14" t="n"/>
       <c r="J50" s="7" t="n"/>
+      <c r="K50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n"/>
@@ -1779,6 +1853,7 @@
       <c r="H51" s="7" t="n"/>
       <c r="I51" s="14" t="n"/>
       <c r="J51" s="7" t="n"/>
+      <c r="K51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n"/>
@@ -1794,6 +1869,7 @@
       <c r="H52" s="7" t="n"/>
       <c r="I52" s="14" t="n"/>
       <c r="J52" s="7" t="n"/>
+      <c r="K52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n"/>
@@ -1809,6 +1885,7 @@
       <c r="H53" s="7" t="n"/>
       <c r="I53" s="14" t="n"/>
       <c r="J53" s="7" t="n"/>
+      <c r="K53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n"/>
@@ -1824,6 +1901,7 @@
       <c r="H54" s="7" t="n"/>
       <c r="I54" s="14" t="n"/>
       <c r="J54" s="7" t="n"/>
+      <c r="K54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n"/>
@@ -1839,6 +1917,7 @@
       <c r="H55" s="7" t="n"/>
       <c r="I55" s="14" t="n"/>
       <c r="J55" s="7" t="n"/>
+      <c r="K55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n"/>
@@ -1854,6 +1933,7 @@
       <c r="H56" s="7" t="n"/>
       <c r="I56" s="14" t="n"/>
       <c r="J56" s="7" t="n"/>
+      <c r="K56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
@@ -1869,6 +1949,7 @@
       <c r="H57" s="7" t="n"/>
       <c r="I57" s="14" t="n"/>
       <c r="J57" s="7" t="n"/>
+      <c r="K57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n"/>
@@ -1884,6 +1965,7 @@
       <c r="H58" s="7" t="n"/>
       <c r="I58" s="14" t="n"/>
       <c r="J58" s="7" t="n"/>
+      <c r="K58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n"/>
@@ -1899,6 +1981,7 @@
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="14" t="n"/>
       <c r="J59" s="7" t="n"/>
+      <c r="K59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n"/>
@@ -1914,6 +1997,7 @@
       <c r="H60" s="7" t="n"/>
       <c r="I60" s="14" t="n"/>
       <c r="J60" s="7" t="n"/>
+      <c r="K60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="n"/>
@@ -1929,6 +2013,7 @@
       <c r="H61" s="7" t="n"/>
       <c r="I61" s="14" t="n"/>
       <c r="J61" s="7" t="n"/>
+      <c r="K61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n"/>
@@ -1944,6 +2029,7 @@
       <c r="H62" s="7" t="n"/>
       <c r="I62" s="14" t="n"/>
       <c r="J62" s="7" t="n"/>
+      <c r="K62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="n"/>
@@ -1959,6 +2045,7 @@
       <c r="H63" s="7" t="n"/>
       <c r="I63" s="14" t="n"/>
       <c r="J63" s="7" t="n"/>
+      <c r="K63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n"/>
@@ -1974,6 +2061,7 @@
       <c r="H64" s="7" t="n"/>
       <c r="I64" s="14" t="n"/>
       <c r="J64" s="7" t="n"/>
+      <c r="K64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="n"/>
@@ -1989,6 +2077,7 @@
       <c r="H65" s="7" t="n"/>
       <c r="I65" s="14" t="n"/>
       <c r="J65" s="7" t="n"/>
+      <c r="K65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n"/>
@@ -2004,6 +2093,7 @@
       <c r="H66" s="7" t="n"/>
       <c r="I66" s="14" t="n"/>
       <c r="J66" s="7" t="n"/>
+      <c r="K66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n"/>
@@ -2019,6 +2109,7 @@
       <c r="H67" s="7" t="n"/>
       <c r="I67" s="14" t="n"/>
       <c r="J67" s="7" t="n"/>
+      <c r="K67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n"/>
@@ -2034,6 +2125,7 @@
       <c r="H68" s="7" t="n"/>
       <c r="I68" s="14" t="n"/>
       <c r="J68" s="7" t="n"/>
+      <c r="K68" s="7" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n"/>
@@ -2049,6 +2141,7 @@
       <c r="H69" s="7" t="n"/>
       <c r="I69" s="14" t="n"/>
       <c r="J69" s="7" t="n"/>
+      <c r="K69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n"/>
@@ -2064,6 +2157,7 @@
       <c r="H70" s="7" t="n"/>
       <c r="I70" s="14" t="n"/>
       <c r="J70" s="7" t="n"/>
+      <c r="K70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="n"/>
@@ -2079,6 +2173,7 @@
       <c r="H71" s="7" t="n"/>
       <c r="I71" s="14" t="n"/>
       <c r="J71" s="7" t="n"/>
+      <c r="K71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n"/>
@@ -2094,6 +2189,7 @@
       <c r="H72" s="7" t="n"/>
       <c r="I72" s="14" t="n"/>
       <c r="J72" s="7" t="n"/>
+      <c r="K72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="n"/>
@@ -2109,6 +2205,7 @@
       <c r="H73" s="7" t="n"/>
       <c r="I73" s="14" t="n"/>
       <c r="J73" s="7" t="n"/>
+      <c r="K73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="n"/>
@@ -2124,6 +2221,7 @@
       <c r="H74" s="7" t="n"/>
       <c r="I74" s="14" t="n"/>
       <c r="J74" s="7" t="n"/>
+      <c r="K74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="n"/>
@@ -2139,6 +2237,7 @@
       <c r="H75" s="7" t="n"/>
       <c r="I75" s="14" t="n"/>
       <c r="J75" s="7" t="n"/>
+      <c r="K75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n"/>
@@ -2154,6 +2253,7 @@
       <c r="H76" s="7" t="n"/>
       <c r="I76" s="14" t="n"/>
       <c r="J76" s="7" t="n"/>
+      <c r="K76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="n"/>
@@ -2169,6 +2269,7 @@
       <c r="H77" s="7" t="n"/>
       <c r="I77" s="14" t="n"/>
       <c r="J77" s="7" t="n"/>
+      <c r="K77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="n"/>
@@ -2184,6 +2285,7 @@
       <c r="H78" s="7" t="n"/>
       <c r="I78" s="14" t="n"/>
       <c r="J78" s="7" t="n"/>
+      <c r="K78" s="7" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="n"/>
@@ -2199,6 +2301,7 @@
       <c r="H79" s="7" t="n"/>
       <c r="I79" s="14" t="n"/>
       <c r="J79" s="7" t="n"/>
+      <c r="K79" s="7" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="n"/>
@@ -2214,6 +2317,7 @@
       <c r="H80" s="7" t="n"/>
       <c r="I80" s="14" t="n"/>
       <c r="J80" s="7" t="n"/>
+      <c r="K80" s="7" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="n"/>
@@ -2229,6 +2333,7 @@
       <c r="H81" s="7" t="n"/>
       <c r="I81" s="14" t="n"/>
       <c r="J81" s="7" t="n"/>
+      <c r="K81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="n"/>
@@ -2244,6 +2349,7 @@
       <c r="H82" s="7" t="n"/>
       <c r="I82" s="14" t="n"/>
       <c r="J82" s="7" t="n"/>
+      <c r="K82" s="7" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="n"/>
@@ -2259,6 +2365,7 @@
       <c r="H83" s="7" t="n"/>
       <c r="I83" s="14" t="n"/>
       <c r="J83" s="7" t="n"/>
+      <c r="K83" s="7" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="n"/>
@@ -2274,6 +2381,7 @@
       <c r="H84" s="7" t="n"/>
       <c r="I84" s="14" t="n"/>
       <c r="J84" s="7" t="n"/>
+      <c r="K84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="n"/>
@@ -2289,6 +2397,7 @@
       <c r="H85" s="7" t="n"/>
       <c r="I85" s="14" t="n"/>
       <c r="J85" s="7" t="n"/>
+      <c r="K85" s="7" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="n"/>
@@ -2304,6 +2413,7 @@
       <c r="H86" s="7" t="n"/>
       <c r="I86" s="14" t="n"/>
       <c r="J86" s="7" t="n"/>
+      <c r="K86" s="7" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="n"/>
@@ -2319,6 +2429,7 @@
       <c r="H87" s="7" t="n"/>
       <c r="I87" s="14" t="n"/>
       <c r="J87" s="7" t="n"/>
+      <c r="K87" s="7" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="n"/>
@@ -2334,6 +2445,7 @@
       <c r="H88" s="7" t="n"/>
       <c r="I88" s="14" t="n"/>
       <c r="J88" s="7" t="n"/>
+      <c r="K88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="n"/>
@@ -2349,6 +2461,7 @@
       <c r="H89" s="7" t="n"/>
       <c r="I89" s="14" t="n"/>
       <c r="J89" s="7" t="n"/>
+      <c r="K89" s="7" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="n"/>
@@ -2364,6 +2477,7 @@
       <c r="H90" s="7" t="n"/>
       <c r="I90" s="14" t="n"/>
       <c r="J90" s="7" t="n"/>
+      <c r="K90" s="7" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="n"/>
@@ -2379,6 +2493,7 @@
       <c r="H91" s="7" t="n"/>
       <c r="I91" s="14" t="n"/>
       <c r="J91" s="7" t="n"/>
+      <c r="K91" s="7" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="n"/>
@@ -2394,6 +2509,7 @@
       <c r="H92" s="7" t="n"/>
       <c r="I92" s="14" t="n"/>
       <c r="J92" s="7" t="n"/>
+      <c r="K92" s="7" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="n"/>
@@ -2409,6 +2525,7 @@
       <c r="H93" s="7" t="n"/>
       <c r="I93" s="14" t="n"/>
       <c r="J93" s="7" t="n"/>
+      <c r="K93" s="7" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="n"/>
@@ -2424,6 +2541,7 @@
       <c r="H94" s="7" t="n"/>
       <c r="I94" s="14" t="n"/>
       <c r="J94" s="7" t="n"/>
+      <c r="K94" s="7" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="n"/>
@@ -2439,6 +2557,7 @@
       <c r="H95" s="7" t="n"/>
       <c r="I95" s="14" t="n"/>
       <c r="J95" s="7" t="n"/>
+      <c r="K95" s="7" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="n"/>
@@ -2454,6 +2573,7 @@
       <c r="H96" s="7" t="n"/>
       <c r="I96" s="14" t="n"/>
       <c r="J96" s="7" t="n"/>
+      <c r="K96" s="7" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="n"/>
@@ -2469,6 +2589,7 @@
       <c r="H97" s="7" t="n"/>
       <c r="I97" s="14" t="n"/>
       <c r="J97" s="7" t="n"/>
+      <c r="K97" s="7" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="n"/>
@@ -2484,6 +2605,7 @@
       <c r="H98" s="7" t="n"/>
       <c r="I98" s="14" t="n"/>
       <c r="J98" s="7" t="n"/>
+      <c r="K98" s="7" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="n"/>
@@ -2499,6 +2621,7 @@
       <c r="H99" s="7" t="n"/>
       <c r="I99" s="14" t="n"/>
       <c r="J99" s="7" t="n"/>
+      <c r="K99" s="7" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="n"/>
@@ -2514,6 +2637,7 @@
       <c r="H100" s="7" t="n"/>
       <c r="I100" s="14" t="n"/>
       <c r="J100" s="7" t="n"/>
+      <c r="K100" s="7" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="n"/>
@@ -2529,6 +2653,7 @@
       <c r="H101" s="7" t="n"/>
       <c r="I101" s="14" t="n"/>
       <c r="J101" s="7" t="n"/>
+      <c r="K101" s="7" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="n"/>
@@ -2544,6 +2669,7 @@
       <c r="H102" s="7" t="n"/>
       <c r="I102" s="14" t="n"/>
       <c r="J102" s="7" t="n"/>
+      <c r="K102" s="7" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="n"/>
@@ -2559,6 +2685,7 @@
       <c r="H103" s="7" t="n"/>
       <c r="I103" s="14" t="n"/>
       <c r="J103" s="7" t="n"/>
+      <c r="K103" s="7" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="n"/>
@@ -2574,6 +2701,7 @@
       <c r="H104" s="7" t="n"/>
       <c r="I104" s="14" t="n"/>
       <c r="J104" s="7" t="n"/>
+      <c r="K104" s="7" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n"/>
@@ -2589,6 +2717,7 @@
       <c r="H105" s="7" t="n"/>
       <c r="I105" s="14" t="n"/>
       <c r="J105" s="7" t="n"/>
+      <c r="K105" s="7" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="n"/>
@@ -2604,6 +2733,7 @@
       <c r="H106" s="7" t="n"/>
       <c r="I106" s="14" t="n"/>
       <c r="J106" s="7" t="n"/>
+      <c r="K106" s="7" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="n"/>
@@ -2619,6 +2749,7 @@
       <c r="H107" s="7" t="n"/>
       <c r="I107" s="14" t="n"/>
       <c r="J107" s="7" t="n"/>
+      <c r="K107" s="7" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="n"/>
@@ -2634,6 +2765,7 @@
       <c r="H108" s="7" t="n"/>
       <c r="I108" s="14" t="n"/>
       <c r="J108" s="7" t="n"/>
+      <c r="K108" s="7" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="n"/>
@@ -2649,6 +2781,7 @@
       <c r="H109" s="7" t="n"/>
       <c r="I109" s="14" t="n"/>
       <c r="J109" s="7" t="n"/>
+      <c r="K109" s="7" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="n"/>
@@ -2664,6 +2797,7 @@
       <c r="H110" s="7" t="n"/>
       <c r="I110" s="14" t="n"/>
       <c r="J110" s="7" t="n"/>
+      <c r="K110" s="7" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="n"/>
@@ -2679,6 +2813,7 @@
       <c r="H111" s="7" t="n"/>
       <c r="I111" s="14" t="n"/>
       <c r="J111" s="7" t="n"/>
+      <c r="K111" s="7" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="n"/>
@@ -2694,6 +2829,7 @@
       <c r="H112" s="7" t="n"/>
       <c r="I112" s="14" t="n"/>
       <c r="J112" s="7" t="n"/>
+      <c r="K112" s="7" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="n"/>
@@ -2709,6 +2845,7 @@
       <c r="H113" s="7" t="n"/>
       <c r="I113" s="14" t="n"/>
       <c r="J113" s="7" t="n"/>
+      <c r="K113" s="7" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="n"/>
@@ -2724,6 +2861,7 @@
       <c r="H114" s="7" t="n"/>
       <c r="I114" s="14" t="n"/>
       <c r="J114" s="7" t="n"/>
+      <c r="K114" s="7" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="n"/>
@@ -2739,6 +2877,7 @@
       <c r="H115" s="7" t="n"/>
       <c r="I115" s="14" t="n"/>
       <c r="J115" s="7" t="n"/>
+      <c r="K115" s="7" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="n"/>
@@ -2754,6 +2893,7 @@
       <c r="H116" s="7" t="n"/>
       <c r="I116" s="14" t="n"/>
       <c r="J116" s="7" t="n"/>
+      <c r="K116" s="7" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="n"/>
@@ -2769,6 +2909,7 @@
       <c r="H117" s="7" t="n"/>
       <c r="I117" s="14" t="n"/>
       <c r="J117" s="7" t="n"/>
+      <c r="K117" s="7" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="n"/>
@@ -2784,6 +2925,7 @@
       <c r="H118" s="7" t="n"/>
       <c r="I118" s="14" t="n"/>
       <c r="J118" s="7" t="n"/>
+      <c r="K118" s="7" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="n"/>
@@ -2799,6 +2941,7 @@
       <c r="H119" s="7" t="n"/>
       <c r="I119" s="14" t="n"/>
       <c r="J119" s="7" t="n"/>
+      <c r="K119" s="7" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="n"/>
@@ -2814,6 +2957,7 @@
       <c r="H120" s="7" t="n"/>
       <c r="I120" s="14" t="n"/>
       <c r="J120" s="7" t="n"/>
+      <c r="K120" s="7" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="n"/>
@@ -2829,6 +2973,7 @@
       <c r="H121" s="7" t="n"/>
       <c r="I121" s="14" t="n"/>
       <c r="J121" s="7" t="n"/>
+      <c r="K121" s="7" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="n"/>
@@ -2844,6 +2989,7 @@
       <c r="H122" s="7" t="n"/>
       <c r="I122" s="14" t="n"/>
       <c r="J122" s="7" t="n"/>
+      <c r="K122" s="7" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="n"/>
@@ -2859,6 +3005,7 @@
       <c r="H123" s="7" t="n"/>
       <c r="I123" s="14" t="n"/>
       <c r="J123" s="7" t="n"/>
+      <c r="K123" s="7" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="n"/>
@@ -2874,6 +3021,7 @@
       <c r="H124" s="7" t="n"/>
       <c r="I124" s="14" t="n"/>
       <c r="J124" s="7" t="n"/>
+      <c r="K124" s="7" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="n"/>
@@ -2889,6 +3037,7 @@
       <c r="H125" s="7" t="n"/>
       <c r="I125" s="14" t="n"/>
       <c r="J125" s="7" t="n"/>
+      <c r="K125" s="7" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="n"/>
@@ -2904,6 +3053,7 @@
       <c r="H126" s="7" t="n"/>
       <c r="I126" s="14" t="n"/>
       <c r="J126" s="7" t="n"/>
+      <c r="K126" s="7" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="n"/>
@@ -2919,6 +3069,7 @@
       <c r="H127" s="7" t="n"/>
       <c r="I127" s="14" t="n"/>
       <c r="J127" s="7" t="n"/>
+      <c r="K127" s="7" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="n"/>
@@ -2934,6 +3085,7 @@
       <c r="H128" s="7" t="n"/>
       <c r="I128" s="14" t="n"/>
       <c r="J128" s="7" t="n"/>
+      <c r="K128" s="7" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="n"/>
@@ -2949,6 +3101,7 @@
       <c r="H129" s="7" t="n"/>
       <c r="I129" s="14" t="n"/>
       <c r="J129" s="7" t="n"/>
+      <c r="K129" s="7" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="n"/>
@@ -2964,6 +3117,7 @@
       <c r="H130" s="7" t="n"/>
       <c r="I130" s="14" t="n"/>
       <c r="J130" s="7" t="n"/>
+      <c r="K130" s="7" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="n"/>
@@ -2979,6 +3133,7 @@
       <c r="H131" s="7" t="n"/>
       <c r="I131" s="14" t="n"/>
       <c r="J131" s="7" t="n"/>
+      <c r="K131" s="7" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="n"/>
@@ -2994,6 +3149,7 @@
       <c r="H132" s="7" t="n"/>
       <c r="I132" s="14" t="n"/>
       <c r="J132" s="7" t="n"/>
+      <c r="K132" s="7" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="n"/>
@@ -3009,6 +3165,7 @@
       <c r="H133" s="7" t="n"/>
       <c r="I133" s="14" t="n"/>
       <c r="J133" s="7" t="n"/>
+      <c r="K133" s="7" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="n"/>
@@ -3024,6 +3181,7 @@
       <c r="H134" s="7" t="n"/>
       <c r="I134" s="14" t="n"/>
       <c r="J134" s="7" t="n"/>
+      <c r="K134" s="7" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="n"/>
@@ -3039,6 +3197,7 @@
       <c r="H135" s="7" t="n"/>
       <c r="I135" s="14" t="n"/>
       <c r="J135" s="7" t="n"/>
+      <c r="K135" s="7" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="n"/>
@@ -3054,6 +3213,7 @@
       <c r="H136" s="7" t="n"/>
       <c r="I136" s="14" t="n"/>
       <c r="J136" s="7" t="n"/>
+      <c r="K136" s="7" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="n"/>
@@ -3069,6 +3229,7 @@
       <c r="H137" s="7" t="n"/>
       <c r="I137" s="14" t="n"/>
       <c r="J137" s="7" t="n"/>
+      <c r="K137" s="7" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="n"/>
@@ -3084,6 +3245,7 @@
       <c r="H138" s="7" t="n"/>
       <c r="I138" s="14" t="n"/>
       <c r="J138" s="7" t="n"/>
+      <c r="K138" s="7" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="n"/>
@@ -3099,6 +3261,7 @@
       <c r="H139" s="7" t="n"/>
       <c r="I139" s="14" t="n"/>
       <c r="J139" s="7" t="n"/>
+      <c r="K139" s="7" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="n"/>
@@ -3114,6 +3277,7 @@
       <c r="H140" s="7" t="n"/>
       <c r="I140" s="14" t="n"/>
       <c r="J140" s="7" t="n"/>
+      <c r="K140" s="7" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="n"/>
@@ -3129,6 +3293,7 @@
       <c r="H141" s="7" t="n"/>
       <c r="I141" s="14" t="n"/>
       <c r="J141" s="7" t="n"/>
+      <c r="K141" s="7" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="n"/>
@@ -3144,6 +3309,7 @@
       <c r="H142" s="7" t="n"/>
       <c r="I142" s="14" t="n"/>
       <c r="J142" s="7" t="n"/>
+      <c r="K142" s="7" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="n"/>
@@ -3159,6 +3325,7 @@
       <c r="H143" s="7" t="n"/>
       <c r="I143" s="14" t="n"/>
       <c r="J143" s="7" t="n"/>
+      <c r="K143" s="7" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="n"/>
@@ -3174,6 +3341,7 @@
       <c r="H144" s="7" t="n"/>
       <c r="I144" s="14" t="n"/>
       <c r="J144" s="7" t="n"/>
+      <c r="K144" s="7" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="n"/>
@@ -3189,6 +3357,7 @@
       <c r="H145" s="7" t="n"/>
       <c r="I145" s="14" t="n"/>
       <c r="J145" s="7" t="n"/>
+      <c r="K145" s="7" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="n"/>
@@ -3204,6 +3373,7 @@
       <c r="H146" s="7" t="n"/>
       <c r="I146" s="14" t="n"/>
       <c r="J146" s="7" t="n"/>
+      <c r="K146" s="7" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="n"/>
@@ -3219,6 +3389,7 @@
       <c r="H147" s="7" t="n"/>
       <c r="I147" s="14" t="n"/>
       <c r="J147" s="7" t="n"/>
+      <c r="K147" s="7" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="n"/>
@@ -3234,6 +3405,7 @@
       <c r="H148" s="7" t="n"/>
       <c r="I148" s="14" t="n"/>
       <c r="J148" s="7" t="n"/>
+      <c r="K148" s="7" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="n"/>
@@ -3249,6 +3421,7 @@
       <c r="H149" s="7" t="n"/>
       <c r="I149" s="14" t="n"/>
       <c r="J149" s="7" t="n"/>
+      <c r="K149" s="7" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="n"/>
@@ -3264,6 +3437,7 @@
       <c r="H150" s="7" t="n"/>
       <c r="I150" s="14" t="n"/>
       <c r="J150" s="7" t="n"/>
+      <c r="K150" s="7" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="n"/>
@@ -3279,6 +3453,7 @@
       <c r="H151" s="7" t="n"/>
       <c r="I151" s="14" t="n"/>
       <c r="J151" s="7" t="n"/>
+      <c r="K151" s="7" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="n"/>
@@ -3294,6 +3469,7 @@
       <c r="H152" s="7" t="n"/>
       <c r="I152" s="14" t="n"/>
       <c r="J152" s="7" t="n"/>
+      <c r="K152" s="7" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="n"/>
@@ -3309,6 +3485,7 @@
       <c r="H153" s="7" t="n"/>
       <c r="I153" s="14" t="n"/>
       <c r="J153" s="7" t="n"/>
+      <c r="K153" s="7" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="n"/>
@@ -3324,6 +3501,7 @@
       <c r="H154" s="7" t="n"/>
       <c r="I154" s="14" t="n"/>
       <c r="J154" s="7" t="n"/>
+      <c r="K154" s="7" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="n"/>
@@ -3339,6 +3517,7 @@
       <c r="H155" s="7" t="n"/>
       <c r="I155" s="14" t="n"/>
       <c r="J155" s="7" t="n"/>
+      <c r="K155" s="7" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="n"/>
@@ -3354,6 +3533,7 @@
       <c r="H156" s="7" t="n"/>
       <c r="I156" s="14" t="n"/>
       <c r="J156" s="7" t="n"/>
+      <c r="K156" s="7" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="n"/>
@@ -3369,6 +3549,7 @@
       <c r="H157" s="7" t="n"/>
       <c r="I157" s="14" t="n"/>
       <c r="J157" s="7" t="n"/>
+      <c r="K157" s="7" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="n"/>
@@ -3384,6 +3565,7 @@
       <c r="H158" s="7" t="n"/>
       <c r="I158" s="14" t="n"/>
       <c r="J158" s="7" t="n"/>
+      <c r="K158" s="7" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="n"/>
@@ -3399,6 +3581,7 @@
       <c r="H159" s="7" t="n"/>
       <c r="I159" s="14" t="n"/>
       <c r="J159" s="7" t="n"/>
+      <c r="K159" s="7" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="n"/>
@@ -3414,6 +3597,7 @@
       <c r="H160" s="7" t="n"/>
       <c r="I160" s="14" t="n"/>
       <c r="J160" s="7" t="n"/>
+      <c r="K160" s="7" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="n"/>
@@ -3429,6 +3613,7 @@
       <c r="H161" s="7" t="n"/>
       <c r="I161" s="14" t="n"/>
       <c r="J161" s="7" t="n"/>
+      <c r="K161" s="7" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="n"/>
@@ -3444,6 +3629,7 @@
       <c r="H162" s="7" t="n"/>
       <c r="I162" s="14" t="n"/>
       <c r="J162" s="7" t="n"/>
+      <c r="K162" s="7" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="n"/>
@@ -3459,6 +3645,7 @@
       <c r="H163" s="7" t="n"/>
       <c r="I163" s="14" t="n"/>
       <c r="J163" s="7" t="n"/>
+      <c r="K163" s="7" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="n"/>
@@ -3474,6 +3661,7 @@
       <c r="H164" s="7" t="n"/>
       <c r="I164" s="14" t="n"/>
       <c r="J164" s="7" t="n"/>
+      <c r="K164" s="7" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="n"/>
@@ -3489,6 +3677,7 @@
       <c r="H165" s="7" t="n"/>
       <c r="I165" s="14" t="n"/>
       <c r="J165" s="7" t="n"/>
+      <c r="K165" s="7" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="n"/>
@@ -3504,6 +3693,7 @@
       <c r="H166" s="7" t="n"/>
       <c r="I166" s="14" t="n"/>
       <c r="J166" s="7" t="n"/>
+      <c r="K166" s="7" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="n"/>
@@ -3519,6 +3709,7 @@
       <c r="H167" s="7" t="n"/>
       <c r="I167" s="14" t="n"/>
       <c r="J167" s="7" t="n"/>
+      <c r="K167" s="7" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="n"/>
@@ -3534,6 +3725,7 @@
       <c r="H168" s="7" t="n"/>
       <c r="I168" s="14" t="n"/>
       <c r="J168" s="7" t="n"/>
+      <c r="K168" s="7" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="n"/>
@@ -3549,6 +3741,7 @@
       <c r="H169" s="7" t="n"/>
       <c r="I169" s="14" t="n"/>
       <c r="J169" s="7" t="n"/>
+      <c r="K169" s="7" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="n"/>
@@ -3564,6 +3757,7 @@
       <c r="H170" s="7" t="n"/>
       <c r="I170" s="14" t="n"/>
       <c r="J170" s="7" t="n"/>
+      <c r="K170" s="7" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="n"/>
@@ -3579,6 +3773,7 @@
       <c r="H171" s="7" t="n"/>
       <c r="I171" s="14" t="n"/>
       <c r="J171" s="7" t="n"/>
+      <c r="K171" s="7" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="n"/>
@@ -3594,6 +3789,7 @@
       <c r="H172" s="7" t="n"/>
       <c r="I172" s="14" t="n"/>
       <c r="J172" s="7" t="n"/>
+      <c r="K172" s="7" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="n"/>
@@ -3609,6 +3805,7 @@
       <c r="H173" s="7" t="n"/>
       <c r="I173" s="14" t="n"/>
       <c r="J173" s="7" t="n"/>
+      <c r="K173" s="7" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="n"/>
@@ -3624,6 +3821,7 @@
       <c r="H174" s="7" t="n"/>
       <c r="I174" s="14" t="n"/>
       <c r="J174" s="7" t="n"/>
+      <c r="K174" s="7" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="n"/>
@@ -3639,6 +3837,7 @@
       <c r="H175" s="7" t="n"/>
       <c r="I175" s="14" t="n"/>
       <c r="J175" s="7" t="n"/>
+      <c r="K175" s="7" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="n"/>
@@ -3654,6 +3853,7 @@
       <c r="H176" s="7" t="n"/>
       <c r="I176" s="14" t="n"/>
       <c r="J176" s="7" t="n"/>
+      <c r="K176" s="7" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="n"/>
@@ -3669,6 +3869,7 @@
       <c r="H177" s="7" t="n"/>
       <c r="I177" s="14" t="n"/>
       <c r="J177" s="7" t="n"/>
+      <c r="K177" s="7" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="n"/>
@@ -3684,6 +3885,7 @@
       <c r="H178" s="7" t="n"/>
       <c r="I178" s="14" t="n"/>
       <c r="J178" s="7" t="n"/>
+      <c r="K178" s="7" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="n"/>
@@ -3699,6 +3901,7 @@
       <c r="H179" s="7" t="n"/>
       <c r="I179" s="14" t="n"/>
       <c r="J179" s="7" t="n"/>
+      <c r="K179" s="7" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="n"/>
@@ -3714,6 +3917,7 @@
       <c r="H180" s="7" t="n"/>
       <c r="I180" s="14" t="n"/>
       <c r="J180" s="7" t="n"/>
+      <c r="K180" s="7" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="n"/>
@@ -3729,6 +3933,7 @@
       <c r="H181" s="7" t="n"/>
       <c r="I181" s="14" t="n"/>
       <c r="J181" s="7" t="n"/>
+      <c r="K181" s="7" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="n"/>
@@ -3744,6 +3949,7 @@
       <c r="H182" s="7" t="n"/>
       <c r="I182" s="14" t="n"/>
       <c r="J182" s="7" t="n"/>
+      <c r="K182" s="7" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="n"/>
@@ -3759,6 +3965,7 @@
       <c r="H183" s="7" t="n"/>
       <c r="I183" s="14" t="n"/>
       <c r="J183" s="7" t="n"/>
+      <c r="K183" s="7" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="n"/>
@@ -3774,6 +3981,7 @@
       <c r="H184" s="7" t="n"/>
       <c r="I184" s="14" t="n"/>
       <c r="J184" s="7" t="n"/>
+      <c r="K184" s="7" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="n"/>
@@ -3789,6 +3997,7 @@
       <c r="H185" s="7" t="n"/>
       <c r="I185" s="14" t="n"/>
       <c r="J185" s="7" t="n"/>
+      <c r="K185" s="7" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="n"/>
@@ -3804,6 +4013,7 @@
       <c r="H186" s="7" t="n"/>
       <c r="I186" s="14" t="n"/>
       <c r="J186" s="7" t="n"/>
+      <c r="K186" s="7" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="n"/>
@@ -3819,6 +4029,7 @@
       <c r="H187" s="7" t="n"/>
       <c r="I187" s="14" t="n"/>
       <c r="J187" s="7" t="n"/>
+      <c r="K187" s="7" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="n"/>
@@ -3834,6 +4045,7 @@
       <c r="H188" s="7" t="n"/>
       <c r="I188" s="14" t="n"/>
       <c r="J188" s="7" t="n"/>
+      <c r="K188" s="7" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="n"/>
@@ -3849,6 +4061,7 @@
       <c r="H189" s="7" t="n"/>
       <c r="I189" s="14" t="n"/>
       <c r="J189" s="7" t="n"/>
+      <c r="K189" s="7" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="n"/>
@@ -3864,6 +4077,7 @@
       <c r="H190" s="7" t="n"/>
       <c r="I190" s="14" t="n"/>
       <c r="J190" s="7" t="n"/>
+      <c r="K190" s="7" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="n"/>
@@ -3879,6 +4093,7 @@
       <c r="H191" s="7" t="n"/>
       <c r="I191" s="14" t="n"/>
       <c r="J191" s="7" t="n"/>
+      <c r="K191" s="7" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="n"/>
@@ -3894,6 +4109,7 @@
       <c r="H192" s="7" t="n"/>
       <c r="I192" s="14" t="n"/>
       <c r="J192" s="7" t="n"/>
+      <c r="K192" s="7" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="n"/>
@@ -3909,6 +4125,7 @@
       <c r="H193" s="7" t="n"/>
       <c r="I193" s="14" t="n"/>
       <c r="J193" s="7" t="n"/>
+      <c r="K193" s="7" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="n"/>
@@ -3924,6 +4141,7 @@
       <c r="H194" s="7" t="n"/>
       <c r="I194" s="14" t="n"/>
       <c r="J194" s="7" t="n"/>
+      <c r="K194" s="7" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="n"/>
@@ -3939,6 +4157,7 @@
       <c r="H195" s="7" t="n"/>
       <c r="I195" s="14" t="n"/>
       <c r="J195" s="7" t="n"/>
+      <c r="K195" s="7" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="n"/>
@@ -3954,6 +4173,7 @@
       <c r="H196" s="7" t="n"/>
       <c r="I196" s="14" t="n"/>
       <c r="J196" s="7" t="n"/>
+      <c r="K196" s="7" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="n"/>
@@ -3969,6 +4189,7 @@
       <c r="H197" s="7" t="n"/>
       <c r="I197" s="14" t="n"/>
       <c r="J197" s="7" t="n"/>
+      <c r="K197" s="7" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="n"/>
@@ -3984,6 +4205,7 @@
       <c r="H198" s="7" t="n"/>
       <c r="I198" s="14" t="n"/>
       <c r="J198" s="7" t="n"/>
+      <c r="K198" s="7" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="n"/>
@@ -3999,6 +4221,7 @@
       <c r="H199" s="7" t="n"/>
       <c r="I199" s="14" t="n"/>
       <c r="J199" s="7" t="n"/>
+      <c r="K199" s="7" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="n"/>
@@ -4014,6 +4237,7 @@
       <c r="H200" s="7" t="n"/>
       <c r="I200" s="14" t="n"/>
       <c r="J200" s="7" t="n"/>
+      <c r="K200" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -4074,7 +4298,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Add required guarantor (поручитель) to contracts
- New/edit contract form now requires guarantor ФИО + телефон before
  the save button enables, alongside the existing client name
  requirement; needs new guarantor_name/guarantor_phone columns
  (SQL provided separately)
- Guarantor shown in the contract detail sheet (name + formatted phone,
  "не указан" for contracts created before this field existed)
- Excel template: added "Поручитель, ФИО"/"Поручитель, телефон"
  columns; import treats a missing guarantor as a non-blocking notice
  (matching the existing "fill in later" philosophy for bulk import)
  rather than rejecting the row, since forcing it there would undercut
  the deliberately relaxed import validation

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/rassrochki_template.xlsx
+++ b/public/rassrochki_template.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B42"/>
+  <dimension ref="B2:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -673,102 +673,137 @@
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>• Строки-примеры выделены курсивом — их можно удалить перед загрузкой.</t>
+          <t>• «Поручитель, ФИО» и «Поручитель, телефон» — на сайте это обязательные поля</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   для каждого договора. Если оставить их пустыми при импорте, договор всё равно</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Вкладка «Платежи» — если по договору уже что-то оплачено:</t>
+          <t xml:space="preserve">   загрузится, но появится замечание — доберите поручителя позже через</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>• По одной строке на каждый оплаченный платёж: ФИО клиента, № платежа</t>
+          <t xml:space="preserve">   «Изменить договор», иначе на самом сайте новый договор создать без него</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   по графику (1 — первый платёж, 2 — второй и т.д.) и дата, когда он</t>
+          <t xml:space="preserve">   не получится.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   был реально оплачен.</t>
+          <t>• Строки-примеры выделены курсивом — их можно удалить перед загрузкой.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>• Колонку «Товар» заполняйте, только если у клиента несколько договоров —</t>
-        </is>
-      </c>
+      <c r="B33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   она нужна, чтобы отличить, к какому именно договору относится платёж.</t>
+          <t>Вкладка «Платежи» — если по договору уже что-то оплачено:</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>• Не оплаченные платежи вносить не нужно — про них ничего писать не надо,</t>
+          <t>• По одной строке на каждый оплаченный платёж: ФИО клиента, № платежа</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   на сайте они и так будут отображаться как «Ожидает» / «Просрочен».</t>
+          <t xml:space="preserve">   по графику (1 — первый платёж, 2 — второй и т.д.) и дата, когда он</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>• Эта вкладка также работает при повторной загрузке — можно отмечать оплаты</t>
+          <t xml:space="preserve">   был реально оплачен.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   и по договорам, которые уже были на сайте раньше (по ФИО и, если нужно,</t>
+          <t>• Колонку «Товар» заполняйте, только если у клиента несколько договоров —</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   товару).</t>
+          <t xml:space="preserve">   она нужна, чтобы отличить, к какому именно договору относится платёж.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>• Не оплаченные платежи вносить не нужно — про них ничего писать не надо,</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>Повторная загрузка не удаляет уже имеющиеся на сайте данные — новые вкладчики,</t>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   на сайте они и так будут отображаться как «Ожидает» / «Просрочен».</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>• Эта вкладка также работает при повторной загрузке — можно отмечать оплаты</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   и по договорам, которые уже были на сайте раньше (по ФИО и, если нужно,</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   товару).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Повторная загрузка не удаляет уже имеющиеся на сайте данные — новые вкладчики,</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>договоры и платежи из файла добавляются к существующим.</t>
         </is>
@@ -939,7 +974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K200"/>
+  <dimension ref="A1:M200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -953,6 +988,8 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1011,6 +1048,16 @@
           <t>Комментарий</t>
         </is>
       </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Поручитель, ФИО</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Поручитель, телефон</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -1055,6 +1102,16 @@
       <c r="K2" s="9" t="inlineStr">
         <is>
           <t>Просил напомнить за неделю до платежа</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>Иванов Пётр Петрович</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>+7 900 222-33-44</t>
         </is>
       </c>
     </row>
@@ -1086,6 +1143,16 @@
       </c>
       <c r="J3" s="9" t="n"/>
       <c r="K3" s="9" t="inlineStr"/>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>Сергеева Анна Викторовна</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>+7 900 555-66-77</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n"/>
@@ -1102,6 +1169,8 @@
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
+      <c r="L4" s="7" t="n"/>
+      <c r="M4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>
@@ -1118,6 +1187,8 @@
       <c r="I5" s="14" t="n"/>
       <c r="J5" s="7" t="n"/>
       <c r="K5" s="7" t="n"/>
+      <c r="L5" s="7" t="n"/>
+      <c r="M5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n"/>
@@ -1134,6 +1205,8 @@
       <c r="I6" s="14" t="n"/>
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+      <c r="M6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -1150,6 +1223,8 @@
       <c r="I7" s="14" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n"/>
@@ -1166,6 +1241,8 @@
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -1182,6 +1259,8 @@
       <c r="I9" s="14" t="n"/>
       <c r="J9" s="7" t="n"/>
       <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -1198,6 +1277,8 @@
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
+      <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -1214,6 +1295,8 @@
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -1230,6 +1313,8 @@
       <c r="I12" s="14" t="n"/>
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="7" t="n"/>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -1246,6 +1331,8 @@
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="7" t="n"/>
       <c r="K13" s="7" t="n"/>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1262,6 +1349,8 @@
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="7" t="n"/>
       <c r="K14" s="7" t="n"/>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1278,6 +1367,8 @@
       <c r="I15" s="14" t="n"/>
       <c r="J15" s="7" t="n"/>
       <c r="K15" s="7" t="n"/>
+      <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -1294,6 +1385,8 @@
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="7" t="n"/>
       <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n"/>
+      <c r="M16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1310,6 +1403,8 @@
       <c r="I17" s="14" t="n"/>
       <c r="J17" s="7" t="n"/>
       <c r="K17" s="7" t="n"/>
+      <c r="L17" s="7" t="n"/>
+      <c r="M17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1326,6 +1421,8 @@
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
+      <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -1342,6 +1439,8 @@
       <c r="I19" s="14" t="n"/>
       <c r="J19" s="7" t="n"/>
       <c r="K19" s="7" t="n"/>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -1358,6 +1457,8 @@
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="7" t="n"/>
       <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -1374,6 +1475,8 @@
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="7" t="n"/>
       <c r="K21" s="7" t="n"/>
+      <c r="L21" s="7" t="n"/>
+      <c r="M21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -1390,6 +1493,8 @@
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="7" t="n"/>
       <c r="K22" s="7" t="n"/>
+      <c r="L22" s="7" t="n"/>
+      <c r="M22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -1406,6 +1511,8 @@
       <c r="I23" s="14" t="n"/>
       <c r="J23" s="7" t="n"/>
       <c r="K23" s="7" t="n"/>
+      <c r="L23" s="7" t="n"/>
+      <c r="M23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -1422,6 +1529,8 @@
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="7" t="n"/>
       <c r="K24" s="7" t="n"/>
+      <c r="L24" s="7" t="n"/>
+      <c r="M24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -1438,6 +1547,8 @@
       <c r="I25" s="14" t="n"/>
       <c r="J25" s="7" t="n"/>
       <c r="K25" s="7" t="n"/>
+      <c r="L25" s="7" t="n"/>
+      <c r="M25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -1454,6 +1565,8 @@
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="7" t="n"/>
       <c r="K26" s="7" t="n"/>
+      <c r="L26" s="7" t="n"/>
+      <c r="M26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -1470,6 +1583,8 @@
       <c r="I27" s="14" t="n"/>
       <c r="J27" s="7" t="n"/>
       <c r="K27" s="7" t="n"/>
+      <c r="L27" s="7" t="n"/>
+      <c r="M27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -1486,6 +1601,8 @@
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="7" t="n"/>
       <c r="K28" s="7" t="n"/>
+      <c r="L28" s="7" t="n"/>
+      <c r="M28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -1502,6 +1619,8 @@
       <c r="I29" s="14" t="n"/>
       <c r="J29" s="7" t="n"/>
       <c r="K29" s="7" t="n"/>
+      <c r="L29" s="7" t="n"/>
+      <c r="M29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -1518,6 +1637,8 @@
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="7" t="n"/>
       <c r="K30" s="7" t="n"/>
+      <c r="L30" s="7" t="n"/>
+      <c r="M30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -1534,6 +1655,8 @@
       <c r="I31" s="14" t="n"/>
       <c r="J31" s="7" t="n"/>
       <c r="K31" s="7" t="n"/>
+      <c r="L31" s="7" t="n"/>
+      <c r="M31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -1550,6 +1673,8 @@
       <c r="I32" s="14" t="n"/>
       <c r="J32" s="7" t="n"/>
       <c r="K32" s="7" t="n"/>
+      <c r="L32" s="7" t="n"/>
+      <c r="M32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -1566,6 +1691,8 @@
       <c r="I33" s="14" t="n"/>
       <c r="J33" s="7" t="n"/>
       <c r="K33" s="7" t="n"/>
+      <c r="L33" s="7" t="n"/>
+      <c r="M33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -1582,6 +1709,8 @@
       <c r="I34" s="14" t="n"/>
       <c r="J34" s="7" t="n"/>
       <c r="K34" s="7" t="n"/>
+      <c r="L34" s="7" t="n"/>
+      <c r="M34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -1598,6 +1727,8 @@
       <c r="I35" s="14" t="n"/>
       <c r="J35" s="7" t="n"/>
       <c r="K35" s="7" t="n"/>
+      <c r="L35" s="7" t="n"/>
+      <c r="M35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -1614,6 +1745,8 @@
       <c r="I36" s="14" t="n"/>
       <c r="J36" s="7" t="n"/>
       <c r="K36" s="7" t="n"/>
+      <c r="L36" s="7" t="n"/>
+      <c r="M36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -1630,6 +1763,8 @@
       <c r="I37" s="14" t="n"/>
       <c r="J37" s="7" t="n"/>
       <c r="K37" s="7" t="n"/>
+      <c r="L37" s="7" t="n"/>
+      <c r="M37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -1646,6 +1781,8 @@
       <c r="I38" s="14" t="n"/>
       <c r="J38" s="7" t="n"/>
       <c r="K38" s="7" t="n"/>
+      <c r="L38" s="7" t="n"/>
+      <c r="M38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
@@ -1662,6 +1799,8 @@
       <c r="I39" s="14" t="n"/>
       <c r="J39" s="7" t="n"/>
       <c r="K39" s="7" t="n"/>
+      <c r="L39" s="7" t="n"/>
+      <c r="M39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n"/>
@@ -1678,6 +1817,8 @@
       <c r="I40" s="14" t="n"/>
       <c r="J40" s="7" t="n"/>
       <c r="K40" s="7" t="n"/>
+      <c r="L40" s="7" t="n"/>
+      <c r="M40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n"/>
@@ -1694,6 +1835,8 @@
       <c r="I41" s="14" t="n"/>
       <c r="J41" s="7" t="n"/>
       <c r="K41" s="7" t="n"/>
+      <c r="L41" s="7" t="n"/>
+      <c r="M41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n"/>
@@ -1710,6 +1853,8 @@
       <c r="I42" s="14" t="n"/>
       <c r="J42" s="7" t="n"/>
       <c r="K42" s="7" t="n"/>
+      <c r="L42" s="7" t="n"/>
+      <c r="M42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n"/>
@@ -1726,6 +1871,8 @@
       <c r="I43" s="14" t="n"/>
       <c r="J43" s="7" t="n"/>
       <c r="K43" s="7" t="n"/>
+      <c r="L43" s="7" t="n"/>
+      <c r="M43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n"/>
@@ -1742,6 +1889,8 @@
       <c r="I44" s="14" t="n"/>
       <c r="J44" s="7" t="n"/>
       <c r="K44" s="7" t="n"/>
+      <c r="L44" s="7" t="n"/>
+      <c r="M44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n"/>
@@ -1758,6 +1907,8 @@
       <c r="I45" s="14" t="n"/>
       <c r="J45" s="7" t="n"/>
       <c r="K45" s="7" t="n"/>
+      <c r="L45" s="7" t="n"/>
+      <c r="M45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n"/>
@@ -1774,6 +1925,8 @@
       <c r="I46" s="14" t="n"/>
       <c r="J46" s="7" t="n"/>
       <c r="K46" s="7" t="n"/>
+      <c r="L46" s="7" t="n"/>
+      <c r="M46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n"/>
@@ -1790,6 +1943,8 @@
       <c r="I47" s="14" t="n"/>
       <c r="J47" s="7" t="n"/>
       <c r="K47" s="7" t="n"/>
+      <c r="L47" s="7" t="n"/>
+      <c r="M47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -1806,6 +1961,8 @@
       <c r="I48" s="14" t="n"/>
       <c r="J48" s="7" t="n"/>
       <c r="K48" s="7" t="n"/>
+      <c r="L48" s="7" t="n"/>
+      <c r="M48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n"/>
@@ -1822,6 +1979,8 @@
       <c r="I49" s="14" t="n"/>
       <c r="J49" s="7" t="n"/>
       <c r="K49" s="7" t="n"/>
+      <c r="L49" s="7" t="n"/>
+      <c r="M49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n"/>
@@ -1838,6 +1997,8 @@
       <c r="I50" s="14" t="n"/>
       <c r="J50" s="7" t="n"/>
       <c r="K50" s="7" t="n"/>
+      <c r="L50" s="7" t="n"/>
+      <c r="M50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n"/>
@@ -1854,6 +2015,8 @@
       <c r="I51" s="14" t="n"/>
       <c r="J51" s="7" t="n"/>
       <c r="K51" s="7" t="n"/>
+      <c r="L51" s="7" t="n"/>
+      <c r="M51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n"/>
@@ -1870,6 +2033,8 @@
       <c r="I52" s="14" t="n"/>
       <c r="J52" s="7" t="n"/>
       <c r="K52" s="7" t="n"/>
+      <c r="L52" s="7" t="n"/>
+      <c r="M52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n"/>
@@ -1886,6 +2051,8 @@
       <c r="I53" s="14" t="n"/>
       <c r="J53" s="7" t="n"/>
       <c r="K53" s="7" t="n"/>
+      <c r="L53" s="7" t="n"/>
+      <c r="M53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n"/>
@@ -1902,6 +2069,8 @@
       <c r="I54" s="14" t="n"/>
       <c r="J54" s="7" t="n"/>
       <c r="K54" s="7" t="n"/>
+      <c r="L54" s="7" t="n"/>
+      <c r="M54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n"/>
@@ -1918,6 +2087,8 @@
       <c r="I55" s="14" t="n"/>
       <c r="J55" s="7" t="n"/>
       <c r="K55" s="7" t="n"/>
+      <c r="L55" s="7" t="n"/>
+      <c r="M55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n"/>
@@ -1934,6 +2105,8 @@
       <c r="I56" s="14" t="n"/>
       <c r="J56" s="7" t="n"/>
       <c r="K56" s="7" t="n"/>
+      <c r="L56" s="7" t="n"/>
+      <c r="M56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
@@ -1950,6 +2123,8 @@
       <c r="I57" s="14" t="n"/>
       <c r="J57" s="7" t="n"/>
       <c r="K57" s="7" t="n"/>
+      <c r="L57" s="7" t="n"/>
+      <c r="M57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n"/>
@@ -1966,6 +2141,8 @@
       <c r="I58" s="14" t="n"/>
       <c r="J58" s="7" t="n"/>
       <c r="K58" s="7" t="n"/>
+      <c r="L58" s="7" t="n"/>
+      <c r="M58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n"/>
@@ -1982,6 +2159,8 @@
       <c r="I59" s="14" t="n"/>
       <c r="J59" s="7" t="n"/>
       <c r="K59" s="7" t="n"/>
+      <c r="L59" s="7" t="n"/>
+      <c r="M59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n"/>
@@ -1998,6 +2177,8 @@
       <c r="I60" s="14" t="n"/>
       <c r="J60" s="7" t="n"/>
       <c r="K60" s="7" t="n"/>
+      <c r="L60" s="7" t="n"/>
+      <c r="M60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="n"/>
@@ -2014,6 +2195,8 @@
       <c r="I61" s="14" t="n"/>
       <c r="J61" s="7" t="n"/>
       <c r="K61" s="7" t="n"/>
+      <c r="L61" s="7" t="n"/>
+      <c r="M61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n"/>
@@ -2030,6 +2213,8 @@
       <c r="I62" s="14" t="n"/>
       <c r="J62" s="7" t="n"/>
       <c r="K62" s="7" t="n"/>
+      <c r="L62" s="7" t="n"/>
+      <c r="M62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="n"/>
@@ -2046,6 +2231,8 @@
       <c r="I63" s="14" t="n"/>
       <c r="J63" s="7" t="n"/>
       <c r="K63" s="7" t="n"/>
+      <c r="L63" s="7" t="n"/>
+      <c r="M63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n"/>
@@ -2062,6 +2249,8 @@
       <c r="I64" s="14" t="n"/>
       <c r="J64" s="7" t="n"/>
       <c r="K64" s="7" t="n"/>
+      <c r="L64" s="7" t="n"/>
+      <c r="M64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="n"/>
@@ -2078,6 +2267,8 @@
       <c r="I65" s="14" t="n"/>
       <c r="J65" s="7" t="n"/>
       <c r="K65" s="7" t="n"/>
+      <c r="L65" s="7" t="n"/>
+      <c r="M65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n"/>
@@ -2094,6 +2285,8 @@
       <c r="I66" s="14" t="n"/>
       <c r="J66" s="7" t="n"/>
       <c r="K66" s="7" t="n"/>
+      <c r="L66" s="7" t="n"/>
+      <c r="M66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n"/>
@@ -2110,6 +2303,8 @@
       <c r="I67" s="14" t="n"/>
       <c r="J67" s="7" t="n"/>
       <c r="K67" s="7" t="n"/>
+      <c r="L67" s="7" t="n"/>
+      <c r="M67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n"/>
@@ -2126,6 +2321,8 @@
       <c r="I68" s="14" t="n"/>
       <c r="J68" s="7" t="n"/>
       <c r="K68" s="7" t="n"/>
+      <c r="L68" s="7" t="n"/>
+      <c r="M68" s="7" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n"/>
@@ -2142,6 +2339,8 @@
       <c r="I69" s="14" t="n"/>
       <c r="J69" s="7" t="n"/>
       <c r="K69" s="7" t="n"/>
+      <c r="L69" s="7" t="n"/>
+      <c r="M69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n"/>
@@ -2158,6 +2357,8 @@
       <c r="I70" s="14" t="n"/>
       <c r="J70" s="7" t="n"/>
       <c r="K70" s="7" t="n"/>
+      <c r="L70" s="7" t="n"/>
+      <c r="M70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="n"/>
@@ -2174,6 +2375,8 @@
       <c r="I71" s="14" t="n"/>
       <c r="J71" s="7" t="n"/>
       <c r="K71" s="7" t="n"/>
+      <c r="L71" s="7" t="n"/>
+      <c r="M71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n"/>
@@ -2190,6 +2393,8 @@
       <c r="I72" s="14" t="n"/>
       <c r="J72" s="7" t="n"/>
       <c r="K72" s="7" t="n"/>
+      <c r="L72" s="7" t="n"/>
+      <c r="M72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="n"/>
@@ -2206,6 +2411,8 @@
       <c r="I73" s="14" t="n"/>
       <c r="J73" s="7" t="n"/>
       <c r="K73" s="7" t="n"/>
+      <c r="L73" s="7" t="n"/>
+      <c r="M73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="n"/>
@@ -2222,6 +2429,8 @@
       <c r="I74" s="14" t="n"/>
       <c r="J74" s="7" t="n"/>
       <c r="K74" s="7" t="n"/>
+      <c r="L74" s="7" t="n"/>
+      <c r="M74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="n"/>
@@ -2238,6 +2447,8 @@
       <c r="I75" s="14" t="n"/>
       <c r="J75" s="7" t="n"/>
       <c r="K75" s="7" t="n"/>
+      <c r="L75" s="7" t="n"/>
+      <c r="M75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n"/>
@@ -2254,6 +2465,8 @@
       <c r="I76" s="14" t="n"/>
       <c r="J76" s="7" t="n"/>
       <c r="K76" s="7" t="n"/>
+      <c r="L76" s="7" t="n"/>
+      <c r="M76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="n"/>
@@ -2270,6 +2483,8 @@
       <c r="I77" s="14" t="n"/>
       <c r="J77" s="7" t="n"/>
       <c r="K77" s="7" t="n"/>
+      <c r="L77" s="7" t="n"/>
+      <c r="M77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="n"/>
@@ -2286,6 +2501,8 @@
       <c r="I78" s="14" t="n"/>
       <c r="J78" s="7" t="n"/>
       <c r="K78" s="7" t="n"/>
+      <c r="L78" s="7" t="n"/>
+      <c r="M78" s="7" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="n"/>
@@ -2302,6 +2519,8 @@
       <c r="I79" s="14" t="n"/>
       <c r="J79" s="7" t="n"/>
       <c r="K79" s="7" t="n"/>
+      <c r="L79" s="7" t="n"/>
+      <c r="M79" s="7" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="n"/>
@@ -2318,6 +2537,8 @@
       <c r="I80" s="14" t="n"/>
       <c r="J80" s="7" t="n"/>
       <c r="K80" s="7" t="n"/>
+      <c r="L80" s="7" t="n"/>
+      <c r="M80" s="7" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="n"/>
@@ -2334,6 +2555,8 @@
       <c r="I81" s="14" t="n"/>
       <c r="J81" s="7" t="n"/>
       <c r="K81" s="7" t="n"/>
+      <c r="L81" s="7" t="n"/>
+      <c r="M81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="n"/>
@@ -2350,6 +2573,8 @@
       <c r="I82" s="14" t="n"/>
       <c r="J82" s="7" t="n"/>
       <c r="K82" s="7" t="n"/>
+      <c r="L82" s="7" t="n"/>
+      <c r="M82" s="7" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="n"/>
@@ -2366,6 +2591,8 @@
       <c r="I83" s="14" t="n"/>
       <c r="J83" s="7" t="n"/>
       <c r="K83" s="7" t="n"/>
+      <c r="L83" s="7" t="n"/>
+      <c r="M83" s="7" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="n"/>
@@ -2382,6 +2609,8 @@
       <c r="I84" s="14" t="n"/>
       <c r="J84" s="7" t="n"/>
       <c r="K84" s="7" t="n"/>
+      <c r="L84" s="7" t="n"/>
+      <c r="M84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="n"/>
@@ -2398,6 +2627,8 @@
       <c r="I85" s="14" t="n"/>
       <c r="J85" s="7" t="n"/>
       <c r="K85" s="7" t="n"/>
+      <c r="L85" s="7" t="n"/>
+      <c r="M85" s="7" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="n"/>
@@ -2414,6 +2645,8 @@
       <c r="I86" s="14" t="n"/>
       <c r="J86" s="7" t="n"/>
       <c r="K86" s="7" t="n"/>
+      <c r="L86" s="7" t="n"/>
+      <c r="M86" s="7" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="n"/>
@@ -2430,6 +2663,8 @@
       <c r="I87" s="14" t="n"/>
       <c r="J87" s="7" t="n"/>
       <c r="K87" s="7" t="n"/>
+      <c r="L87" s="7" t="n"/>
+      <c r="M87" s="7" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="n"/>
@@ -2446,6 +2681,8 @@
       <c r="I88" s="14" t="n"/>
       <c r="J88" s="7" t="n"/>
       <c r="K88" s="7" t="n"/>
+      <c r="L88" s="7" t="n"/>
+      <c r="M88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="n"/>
@@ -2462,6 +2699,8 @@
       <c r="I89" s="14" t="n"/>
       <c r="J89" s="7" t="n"/>
       <c r="K89" s="7" t="n"/>
+      <c r="L89" s="7" t="n"/>
+      <c r="M89" s="7" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="n"/>
@@ -2478,6 +2717,8 @@
       <c r="I90" s="14" t="n"/>
       <c r="J90" s="7" t="n"/>
       <c r="K90" s="7" t="n"/>
+      <c r="L90" s="7" t="n"/>
+      <c r="M90" s="7" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="n"/>
@@ -2494,6 +2735,8 @@
       <c r="I91" s="14" t="n"/>
       <c r="J91" s="7" t="n"/>
       <c r="K91" s="7" t="n"/>
+      <c r="L91" s="7" t="n"/>
+      <c r="M91" s="7" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="n"/>
@@ -2510,6 +2753,8 @@
       <c r="I92" s="14" t="n"/>
       <c r="J92" s="7" t="n"/>
       <c r="K92" s="7" t="n"/>
+      <c r="L92" s="7" t="n"/>
+      <c r="M92" s="7" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="n"/>
@@ -2526,6 +2771,8 @@
       <c r="I93" s="14" t="n"/>
       <c r="J93" s="7" t="n"/>
       <c r="K93" s="7" t="n"/>
+      <c r="L93" s="7" t="n"/>
+      <c r="M93" s="7" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="n"/>
@@ -2542,6 +2789,8 @@
       <c r="I94" s="14" t="n"/>
       <c r="J94" s="7" t="n"/>
       <c r="K94" s="7" t="n"/>
+      <c r="L94" s="7" t="n"/>
+      <c r="M94" s="7" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="n"/>
@@ -2558,6 +2807,8 @@
       <c r="I95" s="14" t="n"/>
       <c r="J95" s="7" t="n"/>
       <c r="K95" s="7" t="n"/>
+      <c r="L95" s="7" t="n"/>
+      <c r="M95" s="7" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="n"/>
@@ -2574,6 +2825,8 @@
       <c r="I96" s="14" t="n"/>
       <c r="J96" s="7" t="n"/>
       <c r="K96" s="7" t="n"/>
+      <c r="L96" s="7" t="n"/>
+      <c r="M96" s="7" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="n"/>
@@ -2590,6 +2843,8 @@
       <c r="I97" s="14" t="n"/>
       <c r="J97" s="7" t="n"/>
       <c r="K97" s="7" t="n"/>
+      <c r="L97" s="7" t="n"/>
+      <c r="M97" s="7" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="n"/>
@@ -2606,6 +2861,8 @@
       <c r="I98" s="14" t="n"/>
       <c r="J98" s="7" t="n"/>
       <c r="K98" s="7" t="n"/>
+      <c r="L98" s="7" t="n"/>
+      <c r="M98" s="7" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="n"/>
@@ -2622,6 +2879,8 @@
       <c r="I99" s="14" t="n"/>
       <c r="J99" s="7" t="n"/>
       <c r="K99" s="7" t="n"/>
+      <c r="L99" s="7" t="n"/>
+      <c r="M99" s="7" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="n"/>
@@ -2638,6 +2897,8 @@
       <c r="I100" s="14" t="n"/>
       <c r="J100" s="7" t="n"/>
       <c r="K100" s="7" t="n"/>
+      <c r="L100" s="7" t="n"/>
+      <c r="M100" s="7" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="n"/>
@@ -2654,6 +2915,8 @@
       <c r="I101" s="14" t="n"/>
       <c r="J101" s="7" t="n"/>
       <c r="K101" s="7" t="n"/>
+      <c r="L101" s="7" t="n"/>
+      <c r="M101" s="7" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="n"/>
@@ -2670,6 +2933,8 @@
       <c r="I102" s="14" t="n"/>
       <c r="J102" s="7" t="n"/>
       <c r="K102" s="7" t="n"/>
+      <c r="L102" s="7" t="n"/>
+      <c r="M102" s="7" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="n"/>
@@ -2686,6 +2951,8 @@
       <c r="I103" s="14" t="n"/>
       <c r="J103" s="7" t="n"/>
       <c r="K103" s="7" t="n"/>
+      <c r="L103" s="7" t="n"/>
+      <c r="M103" s="7" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="n"/>
@@ -2702,6 +2969,8 @@
       <c r="I104" s="14" t="n"/>
       <c r="J104" s="7" t="n"/>
       <c r="K104" s="7" t="n"/>
+      <c r="L104" s="7" t="n"/>
+      <c r="M104" s="7" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n"/>
@@ -2718,6 +2987,8 @@
       <c r="I105" s="14" t="n"/>
       <c r="J105" s="7" t="n"/>
       <c r="K105" s="7" t="n"/>
+      <c r="L105" s="7" t="n"/>
+      <c r="M105" s="7" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="n"/>
@@ -2734,6 +3005,8 @@
       <c r="I106" s="14" t="n"/>
       <c r="J106" s="7" t="n"/>
       <c r="K106" s="7" t="n"/>
+      <c r="L106" s="7" t="n"/>
+      <c r="M106" s="7" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="n"/>
@@ -2750,6 +3023,8 @@
       <c r="I107" s="14" t="n"/>
       <c r="J107" s="7" t="n"/>
       <c r="K107" s="7" t="n"/>
+      <c r="L107" s="7" t="n"/>
+      <c r="M107" s="7" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="n"/>
@@ -2766,6 +3041,8 @@
       <c r="I108" s="14" t="n"/>
       <c r="J108" s="7" t="n"/>
       <c r="K108" s="7" t="n"/>
+      <c r="L108" s="7" t="n"/>
+      <c r="M108" s="7" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="n"/>
@@ -2782,6 +3059,8 @@
       <c r="I109" s="14" t="n"/>
       <c r="J109" s="7" t="n"/>
       <c r="K109" s="7" t="n"/>
+      <c r="L109" s="7" t="n"/>
+      <c r="M109" s="7" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="n"/>
@@ -2798,6 +3077,8 @@
       <c r="I110" s="14" t="n"/>
       <c r="J110" s="7" t="n"/>
       <c r="K110" s="7" t="n"/>
+      <c r="L110" s="7" t="n"/>
+      <c r="M110" s="7" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="n"/>
@@ -2814,6 +3095,8 @@
       <c r="I111" s="14" t="n"/>
       <c r="J111" s="7" t="n"/>
       <c r="K111" s="7" t="n"/>
+      <c r="L111" s="7" t="n"/>
+      <c r="M111" s="7" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="n"/>
@@ -2830,6 +3113,8 @@
       <c r="I112" s="14" t="n"/>
       <c r="J112" s="7" t="n"/>
       <c r="K112" s="7" t="n"/>
+      <c r="L112" s="7" t="n"/>
+      <c r="M112" s="7" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="n"/>
@@ -2846,6 +3131,8 @@
       <c r="I113" s="14" t="n"/>
       <c r="J113" s="7" t="n"/>
       <c r="K113" s="7" t="n"/>
+      <c r="L113" s="7" t="n"/>
+      <c r="M113" s="7" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="n"/>
@@ -2862,6 +3149,8 @@
       <c r="I114" s="14" t="n"/>
       <c r="J114" s="7" t="n"/>
       <c r="K114" s="7" t="n"/>
+      <c r="L114" s="7" t="n"/>
+      <c r="M114" s="7" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="n"/>
@@ -2878,6 +3167,8 @@
       <c r="I115" s="14" t="n"/>
       <c r="J115" s="7" t="n"/>
       <c r="K115" s="7" t="n"/>
+      <c r="L115" s="7" t="n"/>
+      <c r="M115" s="7" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="n"/>
@@ -2894,6 +3185,8 @@
       <c r="I116" s="14" t="n"/>
       <c r="J116" s="7" t="n"/>
       <c r="K116" s="7" t="n"/>
+      <c r="L116" s="7" t="n"/>
+      <c r="M116" s="7" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="n"/>
@@ -2910,6 +3203,8 @@
       <c r="I117" s="14" t="n"/>
       <c r="J117" s="7" t="n"/>
       <c r="K117" s="7" t="n"/>
+      <c r="L117" s="7" t="n"/>
+      <c r="M117" s="7" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="n"/>
@@ -2926,6 +3221,8 @@
       <c r="I118" s="14" t="n"/>
       <c r="J118" s="7" t="n"/>
       <c r="K118" s="7" t="n"/>
+      <c r="L118" s="7" t="n"/>
+      <c r="M118" s="7" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="n"/>
@@ -2942,6 +3239,8 @@
       <c r="I119" s="14" t="n"/>
       <c r="J119" s="7" t="n"/>
       <c r="K119" s="7" t="n"/>
+      <c r="L119" s="7" t="n"/>
+      <c r="M119" s="7" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="n"/>
@@ -2958,6 +3257,8 @@
       <c r="I120" s="14" t="n"/>
       <c r="J120" s="7" t="n"/>
       <c r="K120" s="7" t="n"/>
+      <c r="L120" s="7" t="n"/>
+      <c r="M120" s="7" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="n"/>
@@ -2974,6 +3275,8 @@
       <c r="I121" s="14" t="n"/>
       <c r="J121" s="7" t="n"/>
       <c r="K121" s="7" t="n"/>
+      <c r="L121" s="7" t="n"/>
+      <c r="M121" s="7" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="n"/>
@@ -2990,6 +3293,8 @@
       <c r="I122" s="14" t="n"/>
       <c r="J122" s="7" t="n"/>
       <c r="K122" s="7" t="n"/>
+      <c r="L122" s="7" t="n"/>
+      <c r="M122" s="7" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="n"/>
@@ -3006,6 +3311,8 @@
       <c r="I123" s="14" t="n"/>
       <c r="J123" s="7" t="n"/>
       <c r="K123" s="7" t="n"/>
+      <c r="L123" s="7" t="n"/>
+      <c r="M123" s="7" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="n"/>
@@ -3022,6 +3329,8 @@
       <c r="I124" s="14" t="n"/>
       <c r="J124" s="7" t="n"/>
       <c r="K124" s="7" t="n"/>
+      <c r="L124" s="7" t="n"/>
+      <c r="M124" s="7" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="n"/>
@@ -3038,6 +3347,8 @@
       <c r="I125" s="14" t="n"/>
       <c r="J125" s="7" t="n"/>
       <c r="K125" s="7" t="n"/>
+      <c r="L125" s="7" t="n"/>
+      <c r="M125" s="7" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="n"/>
@@ -3054,6 +3365,8 @@
       <c r="I126" s="14" t="n"/>
       <c r="J126" s="7" t="n"/>
       <c r="K126" s="7" t="n"/>
+      <c r="L126" s="7" t="n"/>
+      <c r="M126" s="7" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="n"/>
@@ -3070,6 +3383,8 @@
       <c r="I127" s="14" t="n"/>
       <c r="J127" s="7" t="n"/>
       <c r="K127" s="7" t="n"/>
+      <c r="L127" s="7" t="n"/>
+      <c r="M127" s="7" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="n"/>
@@ -3086,6 +3401,8 @@
       <c r="I128" s="14" t="n"/>
       <c r="J128" s="7" t="n"/>
       <c r="K128" s="7" t="n"/>
+      <c r="L128" s="7" t="n"/>
+      <c r="M128" s="7" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="n"/>
@@ -3102,6 +3419,8 @@
       <c r="I129" s="14" t="n"/>
       <c r="J129" s="7" t="n"/>
       <c r="K129" s="7" t="n"/>
+      <c r="L129" s="7" t="n"/>
+      <c r="M129" s="7" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="n"/>
@@ -3118,6 +3437,8 @@
       <c r="I130" s="14" t="n"/>
       <c r="J130" s="7" t="n"/>
       <c r="K130" s="7" t="n"/>
+      <c r="L130" s="7" t="n"/>
+      <c r="M130" s="7" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="n"/>
@@ -3134,6 +3455,8 @@
       <c r="I131" s="14" t="n"/>
       <c r="J131" s="7" t="n"/>
       <c r="K131" s="7" t="n"/>
+      <c r="L131" s="7" t="n"/>
+      <c r="M131" s="7" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="n"/>
@@ -3150,6 +3473,8 @@
       <c r="I132" s="14" t="n"/>
       <c r="J132" s="7" t="n"/>
       <c r="K132" s="7" t="n"/>
+      <c r="L132" s="7" t="n"/>
+      <c r="M132" s="7" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="n"/>
@@ -3166,6 +3491,8 @@
       <c r="I133" s="14" t="n"/>
       <c r="J133" s="7" t="n"/>
       <c r="K133" s="7" t="n"/>
+      <c r="L133" s="7" t="n"/>
+      <c r="M133" s="7" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="n"/>
@@ -3182,6 +3509,8 @@
       <c r="I134" s="14" t="n"/>
       <c r="J134" s="7" t="n"/>
       <c r="K134" s="7" t="n"/>
+      <c r="L134" s="7" t="n"/>
+      <c r="M134" s="7" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="n"/>
@@ -3198,6 +3527,8 @@
       <c r="I135" s="14" t="n"/>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
+      <c r="L135" s="7" t="n"/>
+      <c r="M135" s="7" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="n"/>
@@ -3214,6 +3545,8 @@
       <c r="I136" s="14" t="n"/>
       <c r="J136" s="7" t="n"/>
       <c r="K136" s="7" t="n"/>
+      <c r="L136" s="7" t="n"/>
+      <c r="M136" s="7" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="n"/>
@@ -3230,6 +3563,8 @@
       <c r="I137" s="14" t="n"/>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
+      <c r="L137" s="7" t="n"/>
+      <c r="M137" s="7" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="n"/>
@@ -3246,6 +3581,8 @@
       <c r="I138" s="14" t="n"/>
       <c r="J138" s="7" t="n"/>
       <c r="K138" s="7" t="n"/>
+      <c r="L138" s="7" t="n"/>
+      <c r="M138" s="7" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="n"/>
@@ -3262,6 +3599,8 @@
       <c r="I139" s="14" t="n"/>
       <c r="J139" s="7" t="n"/>
       <c r="K139" s="7" t="n"/>
+      <c r="L139" s="7" t="n"/>
+      <c r="M139" s="7" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="n"/>
@@ -3278,6 +3617,8 @@
       <c r="I140" s="14" t="n"/>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
+      <c r="L140" s="7" t="n"/>
+      <c r="M140" s="7" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="n"/>
@@ -3294,6 +3635,8 @@
       <c r="I141" s="14" t="n"/>
       <c r="J141" s="7" t="n"/>
       <c r="K141" s="7" t="n"/>
+      <c r="L141" s="7" t="n"/>
+      <c r="M141" s="7" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="n"/>
@@ -3310,6 +3653,8 @@
       <c r="I142" s="14" t="n"/>
       <c r="J142" s="7" t="n"/>
       <c r="K142" s="7" t="n"/>
+      <c r="L142" s="7" t="n"/>
+      <c r="M142" s="7" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="n"/>
@@ -3326,6 +3671,8 @@
       <c r="I143" s="14" t="n"/>
       <c r="J143" s="7" t="n"/>
       <c r="K143" s="7" t="n"/>
+      <c r="L143" s="7" t="n"/>
+      <c r="M143" s="7" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="n"/>
@@ -3342,6 +3689,8 @@
       <c r="I144" s="14" t="n"/>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
+      <c r="L144" s="7" t="n"/>
+      <c r="M144" s="7" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="n"/>
@@ -3358,6 +3707,8 @@
       <c r="I145" s="14" t="n"/>
       <c r="J145" s="7" t="n"/>
       <c r="K145" s="7" t="n"/>
+      <c r="L145" s="7" t="n"/>
+      <c r="M145" s="7" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="n"/>
@@ -3374,6 +3725,8 @@
       <c r="I146" s="14" t="n"/>
       <c r="J146" s="7" t="n"/>
       <c r="K146" s="7" t="n"/>
+      <c r="L146" s="7" t="n"/>
+      <c r="M146" s="7" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="n"/>
@@ -3390,6 +3743,8 @@
       <c r="I147" s="14" t="n"/>
       <c r="J147" s="7" t="n"/>
       <c r="K147" s="7" t="n"/>
+      <c r="L147" s="7" t="n"/>
+      <c r="M147" s="7" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="n"/>
@@ -3406,6 +3761,8 @@
       <c r="I148" s="14" t="n"/>
       <c r="J148" s="7" t="n"/>
       <c r="K148" s="7" t="n"/>
+      <c r="L148" s="7" t="n"/>
+      <c r="M148" s="7" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="n"/>
@@ -3422,6 +3779,8 @@
       <c r="I149" s="14" t="n"/>
       <c r="J149" s="7" t="n"/>
       <c r="K149" s="7" t="n"/>
+      <c r="L149" s="7" t="n"/>
+      <c r="M149" s="7" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="n"/>
@@ -3438,6 +3797,8 @@
       <c r="I150" s="14" t="n"/>
       <c r="J150" s="7" t="n"/>
       <c r="K150" s="7" t="n"/>
+      <c r="L150" s="7" t="n"/>
+      <c r="M150" s="7" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="n"/>
@@ -3454,6 +3815,8 @@
       <c r="I151" s="14" t="n"/>
       <c r="J151" s="7" t="n"/>
       <c r="K151" s="7" t="n"/>
+      <c r="L151" s="7" t="n"/>
+      <c r="M151" s="7" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="n"/>
@@ -3470,6 +3833,8 @@
       <c r="I152" s="14" t="n"/>
       <c r="J152" s="7" t="n"/>
       <c r="K152" s="7" t="n"/>
+      <c r="L152" s="7" t="n"/>
+      <c r="M152" s="7" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="n"/>
@@ -3486,6 +3851,8 @@
       <c r="I153" s="14" t="n"/>
       <c r="J153" s="7" t="n"/>
       <c r="K153" s="7" t="n"/>
+      <c r="L153" s="7" t="n"/>
+      <c r="M153" s="7" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="n"/>
@@ -3502,6 +3869,8 @@
       <c r="I154" s="14" t="n"/>
       <c r="J154" s="7" t="n"/>
       <c r="K154" s="7" t="n"/>
+      <c r="L154" s="7" t="n"/>
+      <c r="M154" s="7" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="n"/>
@@ -3518,6 +3887,8 @@
       <c r="I155" s="14" t="n"/>
       <c r="J155" s="7" t="n"/>
       <c r="K155" s="7" t="n"/>
+      <c r="L155" s="7" t="n"/>
+      <c r="M155" s="7" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="n"/>
@@ -3534,6 +3905,8 @@
       <c r="I156" s="14" t="n"/>
       <c r="J156" s="7" t="n"/>
       <c r="K156" s="7" t="n"/>
+      <c r="L156" s="7" t="n"/>
+      <c r="M156" s="7" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="n"/>
@@ -3550,6 +3923,8 @@
       <c r="I157" s="14" t="n"/>
       <c r="J157" s="7" t="n"/>
       <c r="K157" s="7" t="n"/>
+      <c r="L157" s="7" t="n"/>
+      <c r="M157" s="7" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="n"/>
@@ -3566,6 +3941,8 @@
       <c r="I158" s="14" t="n"/>
       <c r="J158" s="7" t="n"/>
       <c r="K158" s="7" t="n"/>
+      <c r="L158" s="7" t="n"/>
+      <c r="M158" s="7" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="n"/>
@@ -3582,6 +3959,8 @@
       <c r="I159" s="14" t="n"/>
       <c r="J159" s="7" t="n"/>
       <c r="K159" s="7" t="n"/>
+      <c r="L159" s="7" t="n"/>
+      <c r="M159" s="7" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="n"/>
@@ -3598,6 +3977,8 @@
       <c r="I160" s="14" t="n"/>
       <c r="J160" s="7" t="n"/>
       <c r="K160" s="7" t="n"/>
+      <c r="L160" s="7" t="n"/>
+      <c r="M160" s="7" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="n"/>
@@ -3614,6 +3995,8 @@
       <c r="I161" s="14" t="n"/>
       <c r="J161" s="7" t="n"/>
       <c r="K161" s="7" t="n"/>
+      <c r="L161" s="7" t="n"/>
+      <c r="M161" s="7" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="n"/>
@@ -3630,6 +4013,8 @@
       <c r="I162" s="14" t="n"/>
       <c r="J162" s="7" t="n"/>
       <c r="K162" s="7" t="n"/>
+      <c r="L162" s="7" t="n"/>
+      <c r="M162" s="7" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="n"/>
@@ -3646,6 +4031,8 @@
       <c r="I163" s="14" t="n"/>
       <c r="J163" s="7" t="n"/>
       <c r="K163" s="7" t="n"/>
+      <c r="L163" s="7" t="n"/>
+      <c r="M163" s="7" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="n"/>
@@ -3662,6 +4049,8 @@
       <c r="I164" s="14" t="n"/>
       <c r="J164" s="7" t="n"/>
       <c r="K164" s="7" t="n"/>
+      <c r="L164" s="7" t="n"/>
+      <c r="M164" s="7" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="n"/>
@@ -3678,6 +4067,8 @@
       <c r="I165" s="14" t="n"/>
       <c r="J165" s="7" t="n"/>
       <c r="K165" s="7" t="n"/>
+      <c r="L165" s="7" t="n"/>
+      <c r="M165" s="7" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="n"/>
@@ -3694,6 +4085,8 @@
       <c r="I166" s="14" t="n"/>
       <c r="J166" s="7" t="n"/>
       <c r="K166" s="7" t="n"/>
+      <c r="L166" s="7" t="n"/>
+      <c r="M166" s="7" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="n"/>
@@ -3710,6 +4103,8 @@
       <c r="I167" s="14" t="n"/>
       <c r="J167" s="7" t="n"/>
       <c r="K167" s="7" t="n"/>
+      <c r="L167" s="7" t="n"/>
+      <c r="M167" s="7" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="n"/>
@@ -3726,6 +4121,8 @@
       <c r="I168" s="14" t="n"/>
       <c r="J168" s="7" t="n"/>
       <c r="K168" s="7" t="n"/>
+      <c r="L168" s="7" t="n"/>
+      <c r="M168" s="7" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="n"/>
@@ -3742,6 +4139,8 @@
       <c r="I169" s="14" t="n"/>
       <c r="J169" s="7" t="n"/>
       <c r="K169" s="7" t="n"/>
+      <c r="L169" s="7" t="n"/>
+      <c r="M169" s="7" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="n"/>
@@ -3758,6 +4157,8 @@
       <c r="I170" s="14" t="n"/>
       <c r="J170" s="7" t="n"/>
       <c r="K170" s="7" t="n"/>
+      <c r="L170" s="7" t="n"/>
+      <c r="M170" s="7" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="n"/>
@@ -3774,6 +4175,8 @@
       <c r="I171" s="14" t="n"/>
       <c r="J171" s="7" t="n"/>
       <c r="K171" s="7" t="n"/>
+      <c r="L171" s="7" t="n"/>
+      <c r="M171" s="7" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="n"/>
@@ -3790,6 +4193,8 @@
       <c r="I172" s="14" t="n"/>
       <c r="J172" s="7" t="n"/>
       <c r="K172" s="7" t="n"/>
+      <c r="L172" s="7" t="n"/>
+      <c r="M172" s="7" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="n"/>
@@ -3806,6 +4211,8 @@
       <c r="I173" s="14" t="n"/>
       <c r="J173" s="7" t="n"/>
       <c r="K173" s="7" t="n"/>
+      <c r="L173" s="7" t="n"/>
+      <c r="M173" s="7" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="n"/>
@@ -3822,6 +4229,8 @@
       <c r="I174" s="14" t="n"/>
       <c r="J174" s="7" t="n"/>
       <c r="K174" s="7" t="n"/>
+      <c r="L174" s="7" t="n"/>
+      <c r="M174" s="7" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="n"/>
@@ -3838,6 +4247,8 @@
       <c r="I175" s="14" t="n"/>
       <c r="J175" s="7" t="n"/>
       <c r="K175" s="7" t="n"/>
+      <c r="L175" s="7" t="n"/>
+      <c r="M175" s="7" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="n"/>
@@ -3854,6 +4265,8 @@
       <c r="I176" s="14" t="n"/>
       <c r="J176" s="7" t="n"/>
       <c r="K176" s="7" t="n"/>
+      <c r="L176" s="7" t="n"/>
+      <c r="M176" s="7" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="n"/>
@@ -3870,6 +4283,8 @@
       <c r="I177" s="14" t="n"/>
       <c r="J177" s="7" t="n"/>
       <c r="K177" s="7" t="n"/>
+      <c r="L177" s="7" t="n"/>
+      <c r="M177" s="7" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="n"/>
@@ -3886,6 +4301,8 @@
       <c r="I178" s="14" t="n"/>
       <c r="J178" s="7" t="n"/>
       <c r="K178" s="7" t="n"/>
+      <c r="L178" s="7" t="n"/>
+      <c r="M178" s="7" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="n"/>
@@ -3902,6 +4319,8 @@
       <c r="I179" s="14" t="n"/>
       <c r="J179" s="7" t="n"/>
       <c r="K179" s="7" t="n"/>
+      <c r="L179" s="7" t="n"/>
+      <c r="M179" s="7" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="n"/>
@@ -3918,6 +4337,8 @@
       <c r="I180" s="14" t="n"/>
       <c r="J180" s="7" t="n"/>
       <c r="K180" s="7" t="n"/>
+      <c r="L180" s="7" t="n"/>
+      <c r="M180" s="7" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="n"/>
@@ -3934,6 +4355,8 @@
       <c r="I181" s="14" t="n"/>
       <c r="J181" s="7" t="n"/>
       <c r="K181" s="7" t="n"/>
+      <c r="L181" s="7" t="n"/>
+      <c r="M181" s="7" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="n"/>
@@ -3950,6 +4373,8 @@
       <c r="I182" s="14" t="n"/>
       <c r="J182" s="7" t="n"/>
       <c r="K182" s="7" t="n"/>
+      <c r="L182" s="7" t="n"/>
+      <c r="M182" s="7" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="n"/>
@@ -3966,6 +4391,8 @@
       <c r="I183" s="14" t="n"/>
       <c r="J183" s="7" t="n"/>
       <c r="K183" s="7" t="n"/>
+      <c r="L183" s="7" t="n"/>
+      <c r="M183" s="7" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="n"/>
@@ -3982,6 +4409,8 @@
       <c r="I184" s="14" t="n"/>
       <c r="J184" s="7" t="n"/>
       <c r="K184" s="7" t="n"/>
+      <c r="L184" s="7" t="n"/>
+      <c r="M184" s="7" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="n"/>
@@ -3998,6 +4427,8 @@
       <c r="I185" s="14" t="n"/>
       <c r="J185" s="7" t="n"/>
       <c r="K185" s="7" t="n"/>
+      <c r="L185" s="7" t="n"/>
+      <c r="M185" s="7" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="n"/>
@@ -4014,6 +4445,8 @@
       <c r="I186" s="14" t="n"/>
       <c r="J186" s="7" t="n"/>
       <c r="K186" s="7" t="n"/>
+      <c r="L186" s="7" t="n"/>
+      <c r="M186" s="7" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="n"/>
@@ -4030,6 +4463,8 @@
       <c r="I187" s="14" t="n"/>
       <c r="J187" s="7" t="n"/>
       <c r="K187" s="7" t="n"/>
+      <c r="L187" s="7" t="n"/>
+      <c r="M187" s="7" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="n"/>
@@ -4046,6 +4481,8 @@
       <c r="I188" s="14" t="n"/>
       <c r="J188" s="7" t="n"/>
       <c r="K188" s="7" t="n"/>
+      <c r="L188" s="7" t="n"/>
+      <c r="M188" s="7" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="n"/>
@@ -4062,6 +4499,8 @@
       <c r="I189" s="14" t="n"/>
       <c r="J189" s="7" t="n"/>
       <c r="K189" s="7" t="n"/>
+      <c r="L189" s="7" t="n"/>
+      <c r="M189" s="7" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="n"/>
@@ -4078,6 +4517,8 @@
       <c r="I190" s="14" t="n"/>
       <c r="J190" s="7" t="n"/>
       <c r="K190" s="7" t="n"/>
+      <c r="L190" s="7" t="n"/>
+      <c r="M190" s="7" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="n"/>
@@ -4094,6 +4535,8 @@
       <c r="I191" s="14" t="n"/>
       <c r="J191" s="7" t="n"/>
       <c r="K191" s="7" t="n"/>
+      <c r="L191" s="7" t="n"/>
+      <c r="M191" s="7" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="n"/>
@@ -4110,6 +4553,8 @@
       <c r="I192" s="14" t="n"/>
       <c r="J192" s="7" t="n"/>
       <c r="K192" s="7" t="n"/>
+      <c r="L192" s="7" t="n"/>
+      <c r="M192" s="7" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="n"/>
@@ -4126,6 +4571,8 @@
       <c r="I193" s="14" t="n"/>
       <c r="J193" s="7" t="n"/>
       <c r="K193" s="7" t="n"/>
+      <c r="L193" s="7" t="n"/>
+      <c r="M193" s="7" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="n"/>
@@ -4142,6 +4589,8 @@
       <c r="I194" s="14" t="n"/>
       <c r="J194" s="7" t="n"/>
       <c r="K194" s="7" t="n"/>
+      <c r="L194" s="7" t="n"/>
+      <c r="M194" s="7" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="n"/>
@@ -4158,6 +4607,8 @@
       <c r="I195" s="14" t="n"/>
       <c r="J195" s="7" t="n"/>
       <c r="K195" s="7" t="n"/>
+      <c r="L195" s="7" t="n"/>
+      <c r="M195" s="7" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="n"/>
@@ -4174,6 +4625,8 @@
       <c r="I196" s="14" t="n"/>
       <c r="J196" s="7" t="n"/>
       <c r="K196" s="7" t="n"/>
+      <c r="L196" s="7" t="n"/>
+      <c r="M196" s="7" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="n"/>
@@ -4190,6 +4643,8 @@
       <c r="I197" s="14" t="n"/>
       <c r="J197" s="7" t="n"/>
       <c r="K197" s="7" t="n"/>
+      <c r="L197" s="7" t="n"/>
+      <c r="M197" s="7" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="n"/>
@@ -4206,6 +4661,8 @@
       <c r="I198" s="14" t="n"/>
       <c r="J198" s="7" t="n"/>
       <c r="K198" s="7" t="n"/>
+      <c r="L198" s="7" t="n"/>
+      <c r="M198" s="7" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="n"/>
@@ -4222,6 +4679,8 @@
       <c r="I199" s="14" t="n"/>
       <c r="J199" s="7" t="n"/>
       <c r="K199" s="7" t="n"/>
+      <c r="L199" s="7" t="n"/>
+      <c r="M199" s="7" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="n"/>
@@ -4238,6 +4697,8 @@
       <c r="I200" s="14" t="n"/>
       <c r="J200" s="7" t="n"/>
       <c r="K200" s="7" t="n"/>
+      <c r="L200" s="7" t="n"/>
+      <c r="M200" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>